<commit_message>
Add Discovery Date column, backfilled from oldest known date per row
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="27.88" customWidth="1" style="17" min="1" max="1"/>
@@ -516,9 +516,14 @@
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="0" t="inlineStr">
         <is>
           <t>Publication Date</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Discovery Date</t>
         </is>
       </c>
     </row>
@@ -583,6 +588,9 @@
       <c r="N2" s="18" t="n">
         <v>46162</v>
       </c>
+      <c r="O2" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -642,6 +650,9 @@
         </is>
       </c>
       <c r="M3" s="16" t="n"/>
+      <c r="O3" s="18" t="n">
+        <v>46168</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -697,6 +708,9 @@
           <t>Strong alignment with developer workflows.</t>
         </is>
       </c>
+      <c r="O4" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -752,6 +766,9 @@
           <t>Fast-moving ecosystem.</t>
         </is>
       </c>
+      <c r="O5" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -807,6 +824,9 @@
           <t>Becoming a de facto standard.</t>
         </is>
       </c>
+      <c r="O6" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -869,6 +889,9 @@
       <c r="N7" s="18" t="n">
         <v>45972</v>
       </c>
+      <c r="O7" s="18" t="n">
+        <v>45962</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -931,6 +954,9 @@
         <is>
           <t>Technical guide to the operational life cycle of AI agents, focusing on deployment &amp; security</t>
         </is>
+      </c>
+      <c r="O8" s="18" t="n">
+        <v>45975</v>
       </c>
     </row>
     <row r="9">
@@ -987,6 +1013,9 @@
           <t>Strong enterprise alignment.</t>
         </is>
       </c>
+      <c r="O9" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -1042,6 +1071,9 @@
           <t>Rapidly evolving.</t>
         </is>
       </c>
+      <c r="O10" s="18" t="n">
+        <v>46082</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -1097,6 +1129,9 @@
           <t>Widely used in research.</t>
         </is>
       </c>
+      <c r="O11" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -1152,6 +1187,9 @@
           <t>Strong retrieval-centric design.</t>
         </is>
       </c>
+      <c r="O12" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -1211,6 +1249,9 @@
         <is>
           <t>Strong reproducibility focus.</t>
         </is>
+      </c>
+      <c r="O13" s="18" t="n">
+        <v>46082</v>
       </c>
     </row>
     <row r="14">
@@ -1267,6 +1308,9 @@
           <t>Good hybrid cloud/HPC support.</t>
         </is>
       </c>
+      <c r="O14" s="18" t="n">
+        <v>46082</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -1322,6 +1366,9 @@
           <t>Strong alignment with scientific workflows.</t>
         </is>
       </c>
+      <c r="O15" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -1377,6 +1424,9 @@
           <t>Strong safety posture.</t>
         </is>
       </c>
+      <c r="O16" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -1432,6 +1482,9 @@
           <t>Strong .NET + Python support.</t>
         </is>
       </c>
+      <c r="O17" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -1487,6 +1540,9 @@
           <t>Good for reproducibility.</t>
         </is>
       </c>
+      <c r="O18" s="18" t="n">
+        <v>46082</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -1542,6 +1598,9 @@
           <t>Useful for risk assessment.</t>
         </is>
       </c>
+      <c r="O19" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
@@ -1597,6 +1656,9 @@
           <t>Strong alignment with institutional risk controls.</t>
         </is>
       </c>
+      <c r="O20" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -1652,6 +1714,9 @@
           <t>Widely adopted governance framework.</t>
         </is>
       </c>
+      <c r="O21" s="18" t="n">
+        <v>45992</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -1706,6 +1771,9 @@
           <t>Essential for secure TLAs via PagedAttention and FP8/AWQ optimization.</t>
         </is>
       </c>
+      <c r="O22" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
@@ -1760,6 +1828,9 @@
           <t>Eliminates network dependency errors by cleanly bundling open model weights.</t>
         </is>
       </c>
+      <c r="O23" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -1823,6 +1894,9 @@
           <t>Grammar constraints ensure localized agentic pipelines always return valid JSON/code.</t>
         </is>
       </c>
+      <c r="O24" s="18" t="n">
+        <v>46162</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -1877,6 +1951,9 @@
           <t>Solves local file parsing/RAG bottlenecks entirely within secure client networks.</t>
         </is>
       </c>
+      <c r="O25" s="18" t="n">
+        <v>46113</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -1931,6 +2008,9 @@
           <t>Outlines the exact connected-to-disconnected asset transfer workflow for enterprise GPUs.</t>
         </is>
       </c>
+      <c r="O26" s="18" t="n">
+        <v>46150</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -1985,6 +2065,9 @@
           <t>Built-in vulnerability scanning ensures agent images remain clean behind the firewall.</t>
         </is>
       </c>
+      <c r="O27" s="18" t="n">
+        <v>46150</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
@@ -2039,6 +2122,9 @@
           <t>Moves past simple how-to guides into formal data isolation and local compliance frameworks.</t>
         </is>
       </c>
+      <c r="O28" s="18" t="n">
+        <v>46150</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -2102,6 +2188,9 @@
           <t>Breaks down the "Memory Wall" economics showing an on-prem breakeven velocity of ~4 months.</t>
         </is>
       </c>
+      <c r="O29" s="18" t="n">
+        <v>46054</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
@@ -2160,6 +2249,9 @@
           <t>The Coalition for Secure AI (CoSAI) is an open ecosystem of AI and security experts</t>
         </is>
       </c>
+      <c r="O30" s="18" t="n">
+        <v>46174</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -2222,6 +2314,9 @@
       <c r="N31" s="18" t="n">
         <v>46119</v>
       </c>
+      <c r="O31" s="18" t="n">
+        <v>46119</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -2285,6 +2380,9 @@
           <t>See blog article: https://www.docker.com/blog/the-3cs-a-framework-for-ai-agent-security/</t>
         </is>
       </c>
+      <c r="O32" s="18" t="n">
+        <v>46213</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -2347,6 +2445,9 @@
         <is>
           <t>MIgrated from API Assistants  - now deprecated.</t>
         </is>
+      </c>
+      <c r="O33" s="18" t="n">
+        <v>46212</v>
       </c>
     </row>
     <row r="34">
@@ -4982,7 +5083,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22.13" customWidth="1" style="17" min="2" max="2"/>
@@ -5054,6 +5155,11 @@
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Discovery Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
@@ -5112,6 +5218,9 @@
         <is>
           <t>Stable API surface.</t>
         </is>
+      </c>
+      <c r="N2" s="18" t="n">
+        <v>46150</v>
       </c>
     </row>
   </sheetData>
@@ -5179,7 +5288,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="26.13" customWidth="1" style="17" min="1" max="1"/>
@@ -5242,6 +5351,11 @@
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Discovery Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
@@ -5295,6 +5409,9 @@
           <t>Evaluates State-Of-The-Art agent performance on multi-million line codebases to assess real-world software engineering capabilities.</t>
         </is>
       </c>
+      <c r="L2" s="18" t="n">
+        <v>46216</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -5343,6 +5460,9 @@
           <t>Papers with Code with State-Of-The-Art (SOTA) Codng Agent Benchmarks</t>
         </is>
       </c>
+      <c r="L3" s="18" t="n">
+        <v>46216</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -5391,6 +5511,9 @@
           <t>Addresses limitations of original SWE-bench by focusing on long-horizon, complex, multi-file software engineering tasks.</t>
         </is>
       </c>
+      <c r="L4" s="18" t="n">
+        <v>46216</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -5434,6 +5557,9 @@
           <t>Scalable framework that generates repository-level tasks from live GitHub PRs across 11 programming languages.</t>
         </is>
       </c>
+      <c r="L5" s="18" t="n">
+        <v>46216</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -5480,6 +5606,9 @@
           <t>Benchmarks agents on hard, realistic tasks within terminal/CLI environments.</t>
         </is>
       </c>
+      <c r="L6" s="18" t="n">
+        <v>46216</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -5526,6 +5655,9 @@
           <t>Benchmark specifically for evaluating the code review capabilities of AI agents.</t>
         </is>
       </c>
+      <c r="L7" s="18" t="n">
+        <v>46216</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -5571,6 +5703,9 @@
         <is>
           <t>Isolates the evaluation of repository exploration, context retrieval, and code localization capabilities.</t>
         </is>
+      </c>
+      <c r="L8" s="18" t="n">
+        <v>46216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Standardize Topic Focus separator, add EDAM/NIST vocabulary docs to Dictionary
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -521,7 +521,7 @@
           <t>Publication Date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="0" t="inlineStr">
         <is>
           <t>Discovery Date</t>
         </is>
@@ -567,7 +567,7 @@
       </c>
       <c r="J2" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Implementation, Deployment</t>
+          <t>Architecture; Implementation; Deployment</t>
         </is>
       </c>
       <c r="K2" s="16" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="J3" s="16" t="inlineStr">
         <is>
-          <t>Workflows, Implementation</t>
+          <t>Workflows; Implementation</t>
         </is>
       </c>
       <c r="K3" s="16" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="J4" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Governance, Security</t>
+          <t>Architecture; Governance; Security</t>
         </is>
       </c>
       <c r="K4" s="16" t="inlineStr">
@@ -748,7 +748,7 @@
       </c>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Implementation</t>
+          <t>Architecture; Implementation</t>
         </is>
       </c>
       <c r="K5" s="16" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Governance</t>
+          <t>Architecture; Governance</t>
         </is>
       </c>
       <c r="K6" s="16" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="J7" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Governance</t>
+          <t>Architecture; Governance</t>
         </is>
       </c>
       <c r="K7" s="16" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="J8" s="16" t="inlineStr">
         <is>
-          <t>Implementation, Security, Deployment</t>
+          <t>Implementation; Security; Deployment</t>
         </is>
       </c>
       <c r="K8" s="16" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="J9" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Deployment</t>
+          <t>Architecture; Deployment</t>
         </is>
       </c>
       <c r="K9" s="16" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="J10" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Implementation</t>
+          <t>Architecture; Implementation</t>
         </is>
       </c>
       <c r="K10" s="16" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Implementation</t>
+          <t>Architecture; Implementation</t>
         </is>
       </c>
       <c r="K11" s="16" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="J12" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Governance</t>
+          <t>Architecture; Governance</t>
         </is>
       </c>
       <c r="K12" s="16" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="J13" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Deployment</t>
+          <t>Architecture; Deployment</t>
         </is>
       </c>
       <c r="K13" s="16" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>Implementation, Deployment</t>
+          <t>Implementation; Deployment</t>
         </is>
       </c>
       <c r="K14" s="16" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="J15" s="16" t="inlineStr">
         <is>
-          <t>Implementation, Data Governance</t>
+          <t>Implementation; Data Governance</t>
         </is>
       </c>
       <c r="K15" s="16" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="J16" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Security</t>
+          <t>Architecture; Security</t>
         </is>
       </c>
       <c r="K16" s="16" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Implementation</t>
+          <t>Architecture; Implementation</t>
         </is>
       </c>
       <c r="K17" s="16" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="J18" s="16" t="inlineStr">
         <is>
-          <t>Architecture, Deployment</t>
+          <t>Architecture; Deployment</t>
         </is>
       </c>
       <c r="K18" s="16" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="J22" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Architecture, Implementation, Deployment</t>
+          <t>Self‑hosted AI; Architecture; Implementation; Deployment</t>
         </is>
       </c>
       <c r="K22" s="16" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="J23" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Implementation, Deployment</t>
+          <t>Self‑hosted AI; Implementation; Deployment</t>
         </is>
       </c>
       <c r="K23" s="16" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="J24" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Architecture, Implementation, Deployment</t>
+          <t>Self‑hosted AI; Architecture; Implementation; Deployment</t>
         </is>
       </c>
       <c r="K24" s="16" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="J25" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Implementation, Deployment</t>
+          <t>Self‑hosted AI; Implementation; Deployment</t>
         </is>
       </c>
       <c r="K25" s="16" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="J26" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Implementation, Network Isolation, Infrastructure Security</t>
+          <t>Self‑hosted AI; Implementation; Network Isolation; Infrastructure Security</t>
         </is>
       </c>
       <c r="K26" s="16" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="J27" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Implementation, Network Isolation, Infrastructure Security, Governance</t>
+          <t>Self‑hosted AI; Implementation; Network Isolation; Infrastructure Security; Governance</t>
         </is>
       </c>
       <c r="K27" s="16" t="inlineStr">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="J28" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Infrastructure Security</t>
+          <t>Self‑hosted AI; Infrastructure Security</t>
         </is>
       </c>
       <c r="K28" s="16" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="J29" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI, Architecture, Governance</t>
+          <t>Self‑hosted AI; Architecture; Governance</t>
         </is>
       </c>
       <c r="K29" s="16" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="J30" s="16" t="inlineStr">
         <is>
-          <t>Infrastructure Security, Security</t>
+          <t>Infrastructure Security; Security</t>
         </is>
       </c>
       <c r="K30" s="16" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="J31" s="16" t="inlineStr">
         <is>
-          <t>Infrastructure Security, Security</t>
+          <t>Infrastructure Security; Security</t>
         </is>
       </c>
       <c r="K31" s="16" t="inlineStr">
@@ -2533,7 +2533,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z78"/>
+  <dimension ref="A1:Z81"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="50.38" customWidth="1" style="17" min="1" max="1"/>
@@ -4204,105 +4204,45 @@
       <c r="Z51" s="13" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>This helps research IT teams quickly find relevant material.</t>
-        </is>
-      </c>
-      <c r="B52" s="13" t="n"/>
-      <c r="C52" s="13" t="n"/>
-      <c r="D52" s="13" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
-      <c r="G52" s="13" t="n"/>
-      <c r="H52" s="13" t="n"/>
-      <c r="I52" s="13" t="n"/>
-      <c r="J52" s="13" t="n"/>
-      <c r="K52" s="13" t="n"/>
-      <c r="L52" s="13" t="n"/>
-      <c r="M52" s="13" t="n"/>
-      <c r="N52" s="13" t="n"/>
-      <c r="O52" s="13" t="n"/>
-      <c r="P52" s="13" t="n"/>
-      <c r="Q52" s="13" t="n"/>
-      <c r="R52" s="13" t="n"/>
-      <c r="S52" s="13" t="n"/>
-      <c r="T52" s="13" t="n"/>
-      <c r="U52" s="13" t="n"/>
-      <c r="V52" s="13" t="n"/>
-      <c r="W52" s="13" t="n"/>
-      <c r="X52" s="13" t="n"/>
-      <c r="Y52" s="13" t="n"/>
-      <c r="Z52" s="13" t="n"/>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Data Protection</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Safeguarding sensitive data specifically (EDAM ontology: "Management of sensitive data") -- distinct from the broader "Security" term above. Newly available for Topic Focus.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>9. Relevance to Research Cyberinfrastructure</t>
-        </is>
-      </c>
-      <c r="B53" s="13" t="n"/>
-      <c r="C53" s="13" t="n"/>
-      <c r="D53" s="13" t="n"/>
-      <c r="E53" s="13" t="n"/>
-      <c r="F53" s="13" t="n"/>
-      <c r="G53" s="13" t="n"/>
-      <c r="H53" s="13" t="n"/>
-      <c r="I53" s="13" t="n"/>
-      <c r="J53" s="13" t="n"/>
-      <c r="K53" s="13" t="n"/>
-      <c r="L53" s="13" t="n"/>
-      <c r="M53" s="13" t="n"/>
-      <c r="N53" s="13" t="n"/>
-      <c r="O53" s="13" t="n"/>
-      <c r="P53" s="13" t="n"/>
-      <c r="Q53" s="13" t="n"/>
-      <c r="R53" s="13" t="n"/>
-      <c r="S53" s="13" t="n"/>
-      <c r="T53" s="13" t="n"/>
-      <c r="U53" s="13" t="n"/>
-      <c r="V53" s="13" t="n"/>
-      <c r="W53" s="13" t="n"/>
-      <c r="X53" s="13" t="n"/>
-      <c r="Y53" s="13" t="n"/>
-      <c r="Z53" s="13" t="n"/>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Controlled vocabulary standard: EDAM ontology (Data management branch)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3071 -- "Data governance" and "Workflows" above are EDAM terms (topic_3571, topic_0769). "Data Protection" above is EDAM topic_4044. Also available for future use: FAIR data (topic_4012), Data quality management (topic_3572), Data curation and archival (topic_0219), Data integration and warehousing (topic_3366). Open ontology, not a paywalled standard -- browsable at https://www.ebi.ac.uk/ols4/ontologies/edam</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>A short tag describing why this matters to research platforms:</t>
-        </is>
-      </c>
-      <c r="B54" s="13" t="n"/>
-      <c r="C54" s="13" t="n"/>
-      <c r="D54" s="13" t="n"/>
-      <c r="E54" s="13" t="n"/>
-      <c r="F54" s="13" t="n"/>
-      <c r="G54" s="13" t="n"/>
-      <c r="H54" s="13" t="n"/>
-      <c r="I54" s="13" t="n"/>
-      <c r="J54" s="13" t="n"/>
-      <c r="K54" s="13" t="n"/>
-      <c r="L54" s="13" t="n"/>
-      <c r="M54" s="13" t="n"/>
-      <c r="N54" s="13" t="n"/>
-      <c r="O54" s="13" t="n"/>
-      <c r="P54" s="13" t="n"/>
-      <c r="Q54" s="13" t="n"/>
-      <c r="R54" s="13" t="n"/>
-      <c r="S54" s="13" t="n"/>
-      <c r="T54" s="13" t="n"/>
-      <c r="U54" s="13" t="n"/>
-      <c r="V54" s="13" t="n"/>
-      <c r="W54" s="13" t="n"/>
-      <c r="X54" s="13" t="n"/>
-      <c r="Y54" s="13" t="n"/>
-      <c r="Z54" s="13" t="n"/>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Optional secondary axis: NIST AI RMF 1.0 trustworthy-AI characteristics</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://nvlpubs.nist.gov/nistpubs/ai/NIST.AI.100-1.pdf -- Valid and Reliable, Safe, Secure and Resilient, Accountable and Transparent, Explainable and Interpretable, Privacy-Enhanced, Fair (harmful bias managed). Optional: for AI-trustworthiness framing EDAM doesn't cover. NOTE: NIST's "Fair (harmful bias managed)" is unrelated to EDAM's "FAIR data" (Findable/Accessible/Interoperable/Reusable data principles) despite sharing the word -- do not conflate the two if both are ever used as tags.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Examples:</t>
+          <t>This helps research IT teams quickly find relevant material.</t>
         </is>
       </c>
       <c r="B55" s="13" t="n"/>
@@ -4334,7 +4274,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Workflow orchestration</t>
+          <t>9. Relevance to Research Cyberinfrastructure</t>
         </is>
       </c>
       <c r="B56" s="13" t="n"/>
@@ -4366,7 +4306,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Data portal integration</t>
+          <t>A short tag describing why this matters to research platforms:</t>
         </is>
       </c>
       <c r="B57" s="13" t="n"/>
@@ -4398,7 +4338,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Metadata / provenance</t>
+          <t>Examples:</t>
         </is>
       </c>
       <c r="B58" s="13" t="n"/>
@@ -4430,7 +4370,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Multi‑agent coordination</t>
+          <t>Workflow orchestration</t>
         </is>
       </c>
       <c r="B59" s="13" t="n"/>
@@ -4462,7 +4402,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>HPC / cloud hybrid workflows</t>
+          <t>Data portal integration</t>
         </is>
       </c>
       <c r="B60" s="13" t="n"/>
@@ -4494,7 +4434,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>Reproducibility</t>
+          <t>Metadata / provenance</t>
         </is>
       </c>
       <c r="B61" s="13" t="n"/>
@@ -4526,7 +4466,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>Federated analysis</t>
+          <t>Multi‑agent coordination</t>
         </is>
       </c>
       <c r="B62" s="13" t="n"/>
@@ -4558,7 +4498,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>User‑facing agent interfaces</t>
+          <t>HPC / cloud hybrid workflows</t>
         </is>
       </c>
       <c r="B63" s="13" t="n"/>
@@ -4590,7 +4530,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>9. Maturity Level (Radar Standard)</t>
+          <t>Reproducibility</t>
         </is>
       </c>
       <c r="B64" s="13" t="n"/>
@@ -4622,7 +4562,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Not about the website — about the technology described.</t>
+          <t>Federated analysis</t>
         </is>
       </c>
       <c r="B65" s="13" t="n"/>
@@ -4654,7 +4594,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>User‑facing agent interfaces</t>
         </is>
       </c>
       <c r="B66" s="13" t="n"/>
@@ -4686,7 +4626,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>9. Maturity Level (Radar Standard)</t>
         </is>
       </c>
       <c r="B67" s="13" t="n"/>
@@ -4718,7 +4658,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>Mature</t>
+          <t>Not about the website — about the technology described.</t>
         </is>
       </c>
       <c r="B68" s="13" t="n"/>
@@ -4750,7 +4690,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Deprecated</t>
+          <t>Emerging</t>
         </is>
       </c>
       <c r="B69" s="13" t="n"/>
@@ -4782,7 +4722,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>This helps teams know whether something is stable enough to consider.</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="B70" s="13" t="n"/>
@@ -4814,7 +4754,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>10. Notes / Key Takeaways</t>
+          <t>Mature</t>
         </is>
       </c>
       <c r="B71" s="13" t="n"/>
@@ -4846,7 +4786,7 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>A short free‑text field:</t>
+          <t>Deprecated</t>
         </is>
       </c>
       <c r="B72" s="13" t="n"/>
@@ -4878,7 +4818,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>breaking changes</t>
+          <t>This helps teams know whether something is stable enough to consider.</t>
         </is>
       </c>
       <c r="B73" s="13" t="n"/>
@@ -4910,7 +4850,7 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>important patterns</t>
+          <t>10. Notes / Key Takeaways</t>
         </is>
       </c>
       <c r="B74" s="13" t="n"/>
@@ -4942,7 +4882,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>new capabilities</t>
+          <t>A short free‑text field:</t>
         </is>
       </c>
       <c r="B75" s="13" t="n"/>
@@ -4974,7 +4914,7 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>relevance to agentic workflows</t>
+          <t>breaking changes</t>
         </is>
       </c>
       <c r="B76" s="13" t="n"/>
@@ -5006,7 +4946,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>implications for research platforms</t>
+          <t>important patterns</t>
         </is>
       </c>
       <c r="B77" s="13" t="n"/>
@@ -5038,7 +4978,7 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>This is where institutional knowledge accumulates.</t>
+          <t>new capabilities</t>
         </is>
       </c>
       <c r="B78" s="13" t="n"/>
@@ -5067,6 +5007,102 @@
       <c r="Y78" s="13" t="n"/>
       <c r="Z78" s="13" t="n"/>
     </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>relevance to agentic workflows</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="n"/>
+      <c r="C79" s="13" t="n"/>
+      <c r="D79" s="13" t="n"/>
+      <c r="E79" s="13" t="n"/>
+      <c r="F79" s="13" t="n"/>
+      <c r="G79" s="13" t="n"/>
+      <c r="H79" s="13" t="n"/>
+      <c r="I79" s="13" t="n"/>
+      <c r="J79" s="13" t="n"/>
+      <c r="K79" s="13" t="n"/>
+      <c r="L79" s="13" t="n"/>
+      <c r="M79" s="13" t="n"/>
+      <c r="N79" s="13" t="n"/>
+      <c r="O79" s="13" t="n"/>
+      <c r="P79" s="13" t="n"/>
+      <c r="Q79" s="13" t="n"/>
+      <c r="R79" s="13" t="n"/>
+      <c r="S79" s="13" t="n"/>
+      <c r="T79" s="13" t="n"/>
+      <c r="U79" s="13" t="n"/>
+      <c r="V79" s="13" t="n"/>
+      <c r="W79" s="13" t="n"/>
+      <c r="X79" s="13" t="n"/>
+      <c r="Y79" s="13" t="n"/>
+      <c r="Z79" s="13" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>implications for research platforms</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="n"/>
+      <c r="C80" s="13" t="n"/>
+      <c r="D80" s="13" t="n"/>
+      <c r="E80" s="13" t="n"/>
+      <c r="F80" s="13" t="n"/>
+      <c r="G80" s="13" t="n"/>
+      <c r="H80" s="13" t="n"/>
+      <c r="I80" s="13" t="n"/>
+      <c r="J80" s="13" t="n"/>
+      <c r="K80" s="13" t="n"/>
+      <c r="L80" s="13" t="n"/>
+      <c r="M80" s="13" t="n"/>
+      <c r="N80" s="13" t="n"/>
+      <c r="O80" s="13" t="n"/>
+      <c r="P80" s="13" t="n"/>
+      <c r="Q80" s="13" t="n"/>
+      <c r="R80" s="13" t="n"/>
+      <c r="S80" s="13" t="n"/>
+      <c r="T80" s="13" t="n"/>
+      <c r="U80" s="13" t="n"/>
+      <c r="V80" s="13" t="n"/>
+      <c r="W80" s="13" t="n"/>
+      <c r="X80" s="13" t="n"/>
+      <c r="Y80" s="13" t="n"/>
+      <c r="Z80" s="13" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>This is where institutional knowledge accumulates.</t>
+        </is>
+      </c>
+      <c r="B81" s="13" t="n"/>
+      <c r="C81" s="13" t="n"/>
+      <c r="D81" s="13" t="n"/>
+      <c r="E81" s="13" t="n"/>
+      <c r="F81" s="13" t="n"/>
+      <c r="G81" s="13" t="n"/>
+      <c r="H81" s="13" t="n"/>
+      <c r="I81" s="13" t="n"/>
+      <c r="J81" s="13" t="n"/>
+      <c r="K81" s="13" t="n"/>
+      <c r="L81" s="13" t="n"/>
+      <c r="M81" s="13" t="n"/>
+      <c r="N81" s="13" t="n"/>
+      <c r="O81" s="13" t="n"/>
+      <c r="P81" s="13" t="n"/>
+      <c r="Q81" s="13" t="n"/>
+      <c r="R81" s="13" t="n"/>
+      <c r="S81" s="13" t="n"/>
+      <c r="T81" s="13" t="n"/>
+      <c r="U81" s="13" t="n"/>
+      <c r="V81" s="13" t="n"/>
+      <c r="W81" s="13" t="n"/>
+      <c r="X81" s="13" t="n"/>
+      <c r="Y81" s="13" t="n"/>
+      <c r="Z81" s="13" t="n"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A964">
     <cfRule type="expression" priority="1" dxfId="5">
@@ -5155,7 +5191,7 @@
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="0" t="inlineStr">
         <is>
           <t>Discovery Date</t>
         </is>
@@ -5351,7 +5387,7 @@
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="0" t="inlineStr">
         <is>
           <t>Discovery Date</t>
         </is>

</xml_diff>

<commit_message>
Move prose-like feature values to Notes; add missing-controlled-value check
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -1757,7 +1757,7 @@
       </c>
       <c r="I22" s="16" t="inlineStr">
         <is>
-          <t>Parallel sampling &amp; tool-calling</t>
+          <t>Deployment patterns; Tool Integration</t>
         </is>
       </c>
       <c r="J22" s="16" t="inlineStr">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="M22" s="16" t="inlineStr">
         <is>
-          <t>Essential for secure TLAs via PagedAttention and FP8/AWQ optimization.</t>
+          <t>Essential for secure TLAs via PagedAttention and FP8/AWQ optimization. Capabilities: Parallel sampling &amp; tool-calling.</t>
         </is>
       </c>
       <c r="O22" s="18" t="n">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>Local embedding &amp; zero-config tools</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="J23" s="16" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="M23" s="16" t="inlineStr">
         <is>
-          <t>Eliminates network dependency errors by cleanly bundling open model weights.</t>
+          <t>Eliminates network dependency errors by cleanly bundling open model weights. Capabilities: Local embedding &amp; zero-config tools.</t>
         </is>
       </c>
       <c r="O23" s="18" t="n">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="I24" s="16" t="inlineStr">
         <is>
-          <t>Grammar-based constrained sampling</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="J24" s="16" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>Grammar constraints ensure localized agentic pipelines always return valid JSON/code.</t>
+          <t>Grammar constraints ensure localized agentic pipelines always return valid JSON/code. Capabilities: Grammar-based constrained sampling.</t>
         </is>
       </c>
       <c r="O24" s="18" t="n">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="I25" s="16" t="inlineStr">
         <is>
-          <t>Local RAG pipelines &amp; offline functions</t>
+          <t>Retrieval</t>
         </is>
       </c>
       <c r="J25" s="16" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </c>
       <c r="M25" s="16" t="inlineStr">
         <is>
-          <t>Solves local file parsing/RAG bottlenecks entirely within secure client networks.</t>
+          <t>Solves local file parsing/RAG bottlenecks entirely within secure client networks. Capabilities: Local RAG pipelines &amp; offline functions.</t>
         </is>
       </c>
       <c r="O25" s="18" t="n">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="I26" s="16" t="inlineStr">
         <is>
-          <t>Tensor-parallel caching &amp; optimized tool-calling</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="J26" s="16" t="inlineStr">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="M26" s="16" t="inlineStr">
         <is>
-          <t>Outlines the exact connected-to-disconnected asset transfer workflow for enterprise GPUs.</t>
+          <t>Outlines the exact connected-to-disconnected asset transfer workflow for enterprise GPUs. Capabilities: Tensor-parallel caching &amp; optimized tool-calling.</t>
         </is>
       </c>
       <c r="O26" s="18" t="n">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
-          <t>Artifact version-locking &amp; immutable tags</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="J27" s="16" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="M27" s="16" t="inlineStr">
         <is>
-          <t>Built-in vulnerability scanning ensures agent images remain clean behind the firewall.</t>
+          <t>Built-in vulnerability scanning ensures agent images remain clean behind the firewall. Capabilities: Artifact version-locking &amp; immutable tags.</t>
         </is>
       </c>
       <c r="O27" s="18" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="I28" s="16" t="inlineStr">
         <is>
-          <t>End-to-end local reference applications</t>
+          <t>Deployment patterns; Retrieval</t>
         </is>
       </c>
       <c r="J28" s="16" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="M28" s="16" t="inlineStr">
         <is>
-          <t>Moves past simple how-to guides into formal data isolation and local compliance frameworks.</t>
+          <t>Moves past simple how-to guides into formal data isolation and local compliance frameworks. Capabilities: End-to-end local reference applications.</t>
         </is>
       </c>
       <c r="O28" s="18" t="n">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="I29" s="16" t="inlineStr">
         <is>
-          <t>Hardware performance scaling &amp; VRAM sizing</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="J29" s="16" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="M29" s="16" t="inlineStr">
         <is>
-          <t>Breaks down the "Memory Wall" economics showing an on-prem breakeven velocity of ~4 months.</t>
+          <t>Breaks down the "Memory Wall" economics showing an on-prem breakeven velocity of ~4 months. Capabilities: Hardware performance scaling &amp; VRAM sizing.</t>
         </is>
       </c>
       <c r="O29" s="18" t="n">
@@ -3681,7 +3681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="17" min="1" max="1"/>
@@ -4543,12 +4543,12 @@
     <row r="51">
       <c r="A51" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B51" s="20" t="inlineStr">
         <is>
-          <t>Artifact version-locking &amp; immutable tags</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="C51" s="20" t="inlineStr"/>
@@ -4559,12 +4559,12 @@
     <row r="52">
       <c r="A52" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
-          <t>End-to-end local reference applications</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C52" s="20" t="inlineStr"/>
@@ -4575,31 +4575,51 @@
     <row r="53">
       <c r="A53" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B53" s="20" t="inlineStr">
         <is>
-          <t>Grammar-based constrained sampling</t>
-        </is>
-      </c>
-      <c r="C53" s="20" t="inlineStr"/>
-      <c r="D53" s="20" t="inlineStr"/>
-      <c r="E53" s="20" t="inlineStr"/>
-      <c r="F53" s="20" t="inlineStr"/>
+          <t>Data governance</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>Focuses specifically on the technical protocols, access controls, data-line security, and de-identification standards used to protect the integrity, quality, and privacy of information throughout its lifecycle</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>topic_3571</t>
+        </is>
+      </c>
+      <c r="F53" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3571</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
-          <t>Hardware performance scaling &amp; VRAM sizing</t>
-        </is>
-      </c>
-      <c r="C54" s="20" t="inlineStr"/>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>The overarching organizational policies, compliance frameworks, and capital allocation strategies that dictate how an enterprise manages its broader IT infrastructure, risk tolerances, and vendor choices</t>
+        </is>
+      </c>
       <c r="D54" s="20" t="inlineStr"/>
       <c r="E54" s="20" t="inlineStr"/>
       <c r="F54" s="20" t="inlineStr"/>
@@ -4607,12 +4627,12 @@
     <row r="55">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B55" s="20" t="inlineStr">
         <is>
-          <t>Local RAG pipelines &amp; offline functions</t>
+          <t>Implementation</t>
         </is>
       </c>
       <c r="C55" s="20" t="inlineStr"/>
@@ -4623,15 +4643,19 @@
     <row r="56">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t>Local embedding &amp; zero-config tools</t>
-        </is>
-      </c>
-      <c r="C56" s="20" t="inlineStr"/>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>The tactical, hands-on execution of installing, configuring, provisioning, and launching software or hardware systems within a specific operational environment</t>
+        </is>
+      </c>
       <c r="D56" s="20" t="inlineStr"/>
       <c r="E56" s="20" t="inlineStr"/>
       <c r="F56" s="20" t="inlineStr"/>
@@ -4639,28 +4663,40 @@
     <row r="57">
       <c r="A57" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B57" s="20" t="inlineStr">
         <is>
-          <t>Parallel sampling &amp; tool-calling</t>
+          <t>Workflows</t>
         </is>
       </c>
       <c r="C57" s="20" t="inlineStr"/>
-      <c r="D57" s="20" t="inlineStr"/>
-      <c r="E57" s="20" t="inlineStr"/>
-      <c r="F57" s="20" t="inlineStr"/>
+      <c r="D57" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>topic_0769</t>
+        </is>
+      </c>
+      <c r="F57" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_0769</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B58" s="20" t="inlineStr">
         <is>
-          <t>Tensor-parallel caching &amp; optimized tool-calling</t>
+          <t>Workflow integration</t>
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr"/>
@@ -4676,7 +4712,7 @@
       </c>
       <c r="B59" s="20" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>Model selection</t>
         </is>
       </c>
       <c r="C59" s="20" t="inlineStr"/>
@@ -4692,7 +4728,7 @@
       </c>
       <c r="B60" s="20" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr"/>
@@ -4708,29 +4744,17 @@
       </c>
       <c r="B61" s="20" t="inlineStr">
         <is>
-          <t>Data governance</t>
+          <t>Architecture Compute</t>
         </is>
       </c>
       <c r="C61" s="20" t="inlineStr">
         <is>
-          <t>Focuses specifically on the technical protocols, access controls, data-line security, and de-identification standards used to protect the integrity, quality, and privacy of information throughout its lifecycle</t>
-        </is>
-      </c>
-      <c r="D61" s="20" t="inlineStr">
-        <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>topic_3571</t>
-        </is>
-      </c>
-      <c r="F61" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3571</t>
-        </is>
-      </c>
+          <t>Physical node topologies, hardware constraints, VRAM bounds, and localized compute execution profiles.</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="inlineStr"/>
+      <c r="E61" s="20" t="inlineStr"/>
+      <c r="F61" s="20" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="20" t="inlineStr">
@@ -4740,12 +4764,12 @@
       </c>
       <c r="B62" s="20" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Network Isolation</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
         <is>
-          <t>The overarching organizational policies, compliance frameworks, and capital allocation strategies that dictate how an enterprise manages its broader IT infrastructure, risk tolerances, and vendor choices</t>
+          <t>Non-egress boundaries, air-gapped artifact staging, localized cloud VPC containers, and firewalled local registries.</t>
         </is>
       </c>
       <c r="D62" s="20" t="inlineStr"/>
@@ -4760,10 +4784,14 @@
       </c>
       <c r="B63" s="20" t="inlineStr">
         <is>
-          <t>Implementation</t>
-        </is>
-      </c>
-      <c r="C63" s="20" t="inlineStr"/>
+          <t>Infrastructure Security</t>
+        </is>
+      </c>
+      <c r="C63" s="20" t="inlineStr">
+        <is>
+          <t>For on-prem LLM deployments, it captures the security of the compute stack as well as the data pipelines</t>
+        </is>
+      </c>
       <c r="D63" s="20" t="inlineStr"/>
       <c r="E63" s="20" t="inlineStr"/>
       <c r="F63" s="20" t="inlineStr"/>
@@ -4776,12 +4804,12 @@
       </c>
       <c r="B64" s="20" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Self‑hosted AI</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
-          <t>The tactical, hands-on execution of installing, configuring, provisioning, and launching software or hardware systems within a specific operational environment</t>
+          <t>Self‑hosted, open‑weights models in contrast to API‑based models like OpenAI, Anthropic, or Gemini</t>
         </is>
       </c>
       <c r="D64" s="20" t="inlineStr"/>
@@ -4796,10 +4824,14 @@
       </c>
       <c r="B65" s="20" t="inlineStr">
         <is>
-          <t>Workflows</t>
-        </is>
-      </c>
-      <c r="C65" s="20" t="inlineStr"/>
+          <t>Data Protection</t>
+        </is>
+      </c>
+      <c r="C65" s="20" t="inlineStr">
+        <is>
+          <t>Safeguarding sensitive data specifically. Distinct from the broader Security term.</t>
+        </is>
+      </c>
       <c r="D65" s="20" t="inlineStr">
         <is>
           <t>EDAM</t>
@@ -4807,12 +4839,12 @@
       </c>
       <c r="E65" s="20" t="inlineStr">
         <is>
-          <t>topic_0769</t>
+          <t>topic_4044</t>
         </is>
       </c>
       <c r="F65" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_0769</t>
+          <t>http://edamontology.org/topic_4044</t>
         </is>
       </c>
     </row>
@@ -4824,13 +4856,29 @@
       </c>
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>Workflow integration</t>
-        </is>
-      </c>
-      <c r="C66" s="20" t="inlineStr"/>
-      <c r="D66" s="20" t="inlineStr"/>
-      <c r="E66" s="20" t="inlineStr"/>
-      <c r="F66" s="20" t="inlineStr"/>
+          <t>FAIR data</t>
+        </is>
+      </c>
+      <c r="C66" s="20" t="inlineStr">
+        <is>
+          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
+        </is>
+      </c>
+      <c r="D66" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E66" s="20" t="inlineStr">
+        <is>
+          <t>topic_4012</t>
+        </is>
+      </c>
+      <c r="F66" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_4012</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="20" t="inlineStr">
@@ -4840,13 +4888,25 @@
       </c>
       <c r="B67" s="20" t="inlineStr">
         <is>
-          <t>Model selection</t>
+          <t>Data quality management</t>
         </is>
       </c>
       <c r="C67" s="20" t="inlineStr"/>
-      <c r="D67" s="20" t="inlineStr"/>
-      <c r="E67" s="20" t="inlineStr"/>
-      <c r="F67" s="20" t="inlineStr"/>
+      <c r="D67" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E67" s="20" t="inlineStr">
+        <is>
+          <t>topic_3572</t>
+        </is>
+      </c>
+      <c r="F67" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3572</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="20" t="inlineStr">
@@ -4856,13 +4916,25 @@
       </c>
       <c r="B68" s="20" t="inlineStr">
         <is>
-          <t>Evaluation</t>
+          <t>Data curation and archival</t>
         </is>
       </c>
       <c r="C68" s="20" t="inlineStr"/>
-      <c r="D68" s="20" t="inlineStr"/>
-      <c r="E68" s="20" t="inlineStr"/>
-      <c r="F68" s="20" t="inlineStr"/>
+      <c r="D68" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>topic_0219</t>
+        </is>
+      </c>
+      <c r="F68" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_0219</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="20" t="inlineStr">
@@ -4872,17 +4944,25 @@
       </c>
       <c r="B69" s="20" t="inlineStr">
         <is>
-          <t>Architecture Compute</t>
-        </is>
-      </c>
-      <c r="C69" s="20" t="inlineStr">
-        <is>
-          <t>Physical node topologies, hardware constraints, VRAM bounds, and localized compute execution profiles.</t>
-        </is>
-      </c>
-      <c r="D69" s="20" t="inlineStr"/>
-      <c r="E69" s="20" t="inlineStr"/>
-      <c r="F69" s="20" t="inlineStr"/>
+          <t>Data integration and warehousing</t>
+        </is>
+      </c>
+      <c r="C69" s="20" t="inlineStr"/>
+      <c r="D69" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E69" s="20" t="inlineStr">
+        <is>
+          <t>topic_3366</t>
+        </is>
+      </c>
+      <c r="F69" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3366</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="20" t="inlineStr">
@@ -4892,17 +4972,25 @@
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>Network Isolation</t>
-        </is>
-      </c>
-      <c r="C70" s="20" t="inlineStr">
-        <is>
-          <t>Non-egress boundaries, air-gapped artifact staging, localized cloud VPC containers, and firewalled local registries.</t>
-        </is>
-      </c>
-      <c r="D70" s="20" t="inlineStr"/>
-      <c r="E70" s="20" t="inlineStr"/>
-      <c r="F70" s="20" t="inlineStr"/>
+          <t>Data architecture, analysis and design</t>
+        </is>
+      </c>
+      <c r="C70" s="20" t="inlineStr"/>
+      <c r="D70" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E70" s="20" t="inlineStr">
+        <is>
+          <t>topic_3365</t>
+        </is>
+      </c>
+      <c r="F70" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3365</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="20" t="inlineStr">
@@ -4912,17 +5000,25 @@
       </c>
       <c r="B71" s="20" t="inlineStr">
         <is>
-          <t>Infrastructure Security</t>
-        </is>
-      </c>
-      <c r="C71" s="20" t="inlineStr">
-        <is>
-          <t>For on-prem LLM deployments, it captures the security of the compute stack as well as the data pipelines</t>
-        </is>
-      </c>
-      <c r="D71" s="20" t="inlineStr"/>
-      <c r="E71" s="20" t="inlineStr"/>
-      <c r="F71" s="20" t="inlineStr"/>
+          <t>Data identity and mapping</t>
+        </is>
+      </c>
+      <c r="C71" s="20" t="inlineStr"/>
+      <c r="D71" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E71" s="20" t="inlineStr">
+        <is>
+          <t>topic_3345</t>
+        </is>
+      </c>
+      <c r="F71" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3345</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="20" t="inlineStr">
@@ -4932,17 +5028,25 @@
       </c>
       <c r="B72" s="20" t="inlineStr">
         <is>
-          <t>Self‑hosted AI</t>
-        </is>
-      </c>
-      <c r="C72" s="20" t="inlineStr">
-        <is>
-          <t>Self‑hosted, open‑weights models in contrast to API‑based models like OpenAI, Anthropic, or Gemini</t>
-        </is>
-      </c>
-      <c r="D72" s="20" t="inlineStr"/>
-      <c r="E72" s="20" t="inlineStr"/>
-      <c r="F72" s="20" t="inlineStr"/>
+          <t>Data rescue</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr"/>
+      <c r="D72" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E72" s="20" t="inlineStr">
+        <is>
+          <t>topic_4011</t>
+        </is>
+      </c>
+      <c r="F72" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_4011</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="20" t="inlineStr">
@@ -4952,29 +5056,21 @@
       </c>
       <c r="B73" s="20" t="inlineStr">
         <is>
-          <t>Data Protection</t>
+          <t>Valid and Reliable</t>
         </is>
       </c>
       <c r="C73" s="20" t="inlineStr">
         <is>
-          <t>Safeguarding sensitive data specifically. Distinct from the broader Security term.</t>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
         </is>
       </c>
       <c r="D73" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E73" s="20" t="inlineStr">
-        <is>
-          <t>topic_4044</t>
-        </is>
-      </c>
-      <c r="F73" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_4044</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E73" s="20" t="inlineStr"/>
+      <c r="F73" s="20" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="20" t="inlineStr">
@@ -4984,29 +5080,21 @@
       </c>
       <c r="B74" s="20" t="inlineStr">
         <is>
-          <t>FAIR data</t>
+          <t>Safe</t>
         </is>
       </c>
       <c r="C74" s="20" t="inlineStr">
         <is>
-          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
         </is>
       </c>
       <c r="D74" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E74" s="20" t="inlineStr">
-        <is>
-          <t>topic_4012</t>
-        </is>
-      </c>
-      <c r="F74" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_4012</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E74" s="20" t="inlineStr"/>
+      <c r="F74" s="20" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="20" t="inlineStr">
@@ -5016,25 +5104,21 @@
       </c>
       <c r="B75" s="20" t="inlineStr">
         <is>
-          <t>Data quality management</t>
-        </is>
-      </c>
-      <c r="C75" s="20" t="inlineStr"/>
+          <t>Secure and Resilient</t>
+        </is>
+      </c>
+      <c r="C75" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D75" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E75" s="20" t="inlineStr">
-        <is>
-          <t>topic_3572</t>
-        </is>
-      </c>
-      <c r="F75" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3572</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E75" s="20" t="inlineStr"/>
+      <c r="F75" s="20" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="20" t="inlineStr">
@@ -5044,25 +5128,21 @@
       </c>
       <c r="B76" s="20" t="inlineStr">
         <is>
-          <t>Data curation and archival</t>
-        </is>
-      </c>
-      <c r="C76" s="20" t="inlineStr"/>
+          <t>Accountable and Transparent</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D76" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E76" s="20" t="inlineStr">
-        <is>
-          <t>topic_0219</t>
-        </is>
-      </c>
-      <c r="F76" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_0219</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E76" s="20" t="inlineStr"/>
+      <c r="F76" s="20" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="20" t="inlineStr">
@@ -5072,25 +5152,21 @@
       </c>
       <c r="B77" s="20" t="inlineStr">
         <is>
-          <t>Data integration and warehousing</t>
-        </is>
-      </c>
-      <c r="C77" s="20" t="inlineStr"/>
+          <t>Explainable and Interpretable</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D77" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E77" s="20" t="inlineStr">
-        <is>
-          <t>topic_3366</t>
-        </is>
-      </c>
-      <c r="F77" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3366</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E77" s="20" t="inlineStr"/>
+      <c r="F77" s="20" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="20" t="inlineStr">
@@ -5100,25 +5176,21 @@
       </c>
       <c r="B78" s="20" t="inlineStr">
         <is>
-          <t>Data architecture, analysis and design</t>
-        </is>
-      </c>
-      <c r="C78" s="20" t="inlineStr"/>
+          <t>Privacy-Enhanced</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D78" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E78" s="20" t="inlineStr">
-        <is>
-          <t>topic_3365</t>
-        </is>
-      </c>
-      <c r="F78" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3365</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E78" s="20" t="inlineStr"/>
+      <c r="F78" s="20" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="20" t="inlineStr">
@@ -5128,285 +5200,85 @@
       </c>
       <c r="B79" s="20" t="inlineStr">
         <is>
-          <t>Data identity and mapping</t>
-        </is>
-      </c>
-      <c r="C79" s="20" t="inlineStr"/>
+          <t>Fair (harmful bias managed)</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic: algorithmic non-discrimination. NOT the same as 'FAIR data'.</t>
+        </is>
+      </c>
       <c r="D79" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E79" s="20" t="inlineStr">
-        <is>
-          <t>topic_3345</t>
-        </is>
-      </c>
-      <c r="F79" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3345</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E79" s="20" t="inlineStr"/>
+      <c r="F79" s="20" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B80" s="20" t="inlineStr">
         <is>
-          <t>Data rescue</t>
+          <t>Emerging</t>
         </is>
       </c>
       <c r="C80" s="20" t="inlineStr"/>
-      <c r="D80" s="20" t="inlineStr">
-        <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E80" s="20" t="inlineStr">
-        <is>
-          <t>topic_4011</t>
-        </is>
-      </c>
-      <c r="F80" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_4011</t>
-        </is>
-      </c>
+      <c r="D80" s="20" t="inlineStr"/>
+      <c r="E80" s="20" t="inlineStr"/>
+      <c r="F80" s="20" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B81" s="20" t="inlineStr">
         <is>
-          <t>Valid and Reliable</t>
-        </is>
-      </c>
-      <c r="C81" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D81" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="C81" s="20" t="inlineStr"/>
+      <c r="D81" s="20" t="inlineStr"/>
       <c r="E81" s="20" t="inlineStr"/>
       <c r="F81" s="20" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B82" s="20" t="inlineStr">
         <is>
-          <t>Safe</t>
-        </is>
-      </c>
-      <c r="C82" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D82" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="C82" s="20" t="inlineStr"/>
+      <c r="D82" s="20" t="inlineStr"/>
       <c r="E82" s="20" t="inlineStr"/>
       <c r="F82" s="20" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B83" s="20" t="inlineStr">
         <is>
-          <t>Secure and Resilient</t>
-        </is>
-      </c>
-      <c r="C83" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D83" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Deprecated</t>
+        </is>
+      </c>
+      <c r="C83" s="20" t="inlineStr"/>
+      <c r="D83" s="20" t="inlineStr"/>
       <c r="E83" s="20" t="inlineStr"/>
       <c r="F83" s="20" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="20" t="inlineStr">
-        <is>
-          <t>Topic Focus</t>
-        </is>
-      </c>
-      <c r="B84" s="20" t="inlineStr">
-        <is>
-          <t>Accountable and Transparent</t>
-        </is>
-      </c>
-      <c r="C84" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D84" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
-      <c r="E84" s="20" t="inlineStr"/>
-      <c r="F84" s="20" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="20" t="inlineStr">
-        <is>
-          <t>Topic Focus</t>
-        </is>
-      </c>
-      <c r="B85" s="20" t="inlineStr">
-        <is>
-          <t>Explainable and Interpretable</t>
-        </is>
-      </c>
-      <c r="C85" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D85" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
-      <c r="E85" s="20" t="inlineStr"/>
-      <c r="F85" s="20" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="20" t="inlineStr">
-        <is>
-          <t>Topic Focus</t>
-        </is>
-      </c>
-      <c r="B86" s="20" t="inlineStr">
-        <is>
-          <t>Privacy-Enhanced</t>
-        </is>
-      </c>
-      <c r="C86" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D86" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
-      <c r="E86" s="20" t="inlineStr"/>
-      <c r="F86" s="20" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="20" t="inlineStr">
-        <is>
-          <t>Topic Focus</t>
-        </is>
-      </c>
-      <c r="B87" s="20" t="inlineStr">
-        <is>
-          <t>Fair (harmful bias managed)</t>
-        </is>
-      </c>
-      <c r="C87" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic: algorithmic non-discrimination. NOT the same as 'FAIR data'.</t>
-        </is>
-      </c>
-      <c r="D87" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
-      <c r="E87" s="20" t="inlineStr"/>
-      <c r="F87" s="20" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B88" s="20" t="inlineStr">
-        <is>
-          <t>Emerging</t>
-        </is>
-      </c>
-      <c r="C88" s="20" t="inlineStr"/>
-      <c r="D88" s="20" t="inlineStr"/>
-      <c r="E88" s="20" t="inlineStr"/>
-      <c r="F88" s="20" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B89" s="20" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="C89" s="20" t="inlineStr"/>
-      <c r="D89" s="20" t="inlineStr"/>
-      <c r="E89" s="20" t="inlineStr"/>
-      <c r="F89" s="20" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B90" s="20" t="inlineStr">
-        <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="C90" s="20" t="inlineStr"/>
-      <c r="D90" s="20" t="inlineStr"/>
-      <c r="E90" s="20" t="inlineStr"/>
-      <c r="F90" s="20" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B91" s="20" t="inlineStr">
-        <is>
-          <t>Deprecated</t>
-        </is>
-      </c>
-      <c r="C91" s="20" t="inlineStr"/>
-      <c r="D91" s="20" t="inlineStr"/>
-      <c r="E91" s="20" t="inlineStr"/>
-      <c r="F91" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix stale verification leak: xlsx_to_json.py now writes back blanked cells
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -1337,9 +1337,7 @@
           <t>Project Jupyter</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>46150</v>
-      </c>
+      <c r="D15" s="6" t="n"/>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="7" t="n">
         <v>46113</v>
@@ -1352,7 +1350,7 @@
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>Notebook Agents; Tool Integration</t>
+          <t>Notebook Agents; Workflow Automation</t>
         </is>
       </c>
       <c r="J15" s="16" t="inlineStr">
@@ -1743,9 +1741,7 @@
           <t>vLLM Project Team</t>
         </is>
       </c>
-      <c r="D22" s="6" t="n">
-        <v>46150</v>
-      </c>
+      <c r="D22" s="6" t="n"/>
       <c r="F22" s="7" t="n">
         <v>46113</v>
       </c>
@@ -1757,7 +1753,7 @@
       </c>
       <c r="I22" s="16" t="inlineStr">
         <is>
-          <t>Deployment patterns; Tool Integration</t>
+          <t>Deployment patterns; Tools</t>
         </is>
       </c>
       <c r="J22" s="16" t="inlineStr">
@@ -1857,14 +1853,8 @@
           <t>Georgi Gerganov</t>
         </is>
       </c>
-      <c r="D24" s="6" t="n">
-        <v>46162</v>
-      </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>Paty Buendia</t>
-        </is>
-      </c>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="16" t="n"/>
       <c r="F24" s="14" t="n">
         <v>46162</v>
       </c>
@@ -1980,9 +1970,7 @@
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="D26" s="6" t="n">
-        <v>46150</v>
-      </c>
+      <c r="D26" s="6" t="n"/>
       <c r="F26" s="16" t="n">
         <v>2026</v>
       </c>
@@ -1999,7 +1987,7 @@
       </c>
       <c r="J26" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI; Implementation; Network Isolation; Infrastructure Security</t>
+          <t>Self‑hosted AI; Architecture Compute; Implementation; Network Isolation; Infrastructure Security</t>
         </is>
       </c>
       <c r="K26" s="16" t="inlineStr">
@@ -2151,14 +2139,8 @@
           <t>Lenovo Press</t>
         </is>
       </c>
-      <c r="D29" s="6" t="n">
-        <v>46157</v>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>Paty Buendia</t>
-        </is>
-      </c>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="16" t="n"/>
       <c r="F29" s="7" t="n">
         <v>46054</v>
       </c>
@@ -3681,7 +3663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="17" min="1" max="1"/>
@@ -4244,7 +4226,7 @@
       </c>
       <c r="B33" s="20" t="inlineStr">
         <is>
-          <t>Tool Integration</t>
+          <t>Tool-Ready Endpoints</t>
         </is>
       </c>
       <c r="C33" s="20" t="inlineStr"/>
@@ -4260,7 +4242,7 @@
       </c>
       <c r="B34" s="20" t="inlineStr">
         <is>
-          <t>Tool-Ready Endpoints</t>
+          <t>Coding Agents</t>
         </is>
       </c>
       <c r="C34" s="20" t="inlineStr"/>
@@ -4276,7 +4258,7 @@
       </c>
       <c r="B35" s="20" t="inlineStr">
         <is>
-          <t>Coding Agents</t>
+          <t>Notebook Agents</t>
         </is>
       </c>
       <c r="C35" s="20" t="inlineStr"/>
@@ -4292,7 +4274,7 @@
       </c>
       <c r="B36" s="20" t="inlineStr">
         <is>
-          <t>Notebook Agents</t>
+          <t>Workflow Agents</t>
         </is>
       </c>
       <c r="C36" s="20" t="inlineStr"/>
@@ -4308,7 +4290,7 @@
       </c>
       <c r="B37" s="20" t="inlineStr">
         <is>
-          <t>Workflow Agents</t>
+          <t>Workflow Automation</t>
         </is>
       </c>
       <c r="C37" s="20" t="inlineStr"/>
@@ -4324,7 +4306,7 @@
       </c>
       <c r="B38" s="20" t="inlineStr">
         <is>
-          <t>Workflow Automation</t>
+          <t>Orchestration</t>
         </is>
       </c>
       <c r="C38" s="20" t="inlineStr"/>
@@ -4340,7 +4322,7 @@
       </c>
       <c r="B39" s="20" t="inlineStr">
         <is>
-          <t>Orchestration</t>
+          <t>Triggers</t>
         </is>
       </c>
       <c r="C39" s="20" t="inlineStr"/>
@@ -4356,7 +4338,7 @@
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>Triggers</t>
+          <t>Retrieval</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr"/>
@@ -4372,7 +4354,7 @@
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
-          <t>Retrieval</t>
+          <t>Retrieval Agents</t>
         </is>
       </c>
       <c r="C41" s="20" t="inlineStr"/>
@@ -4388,7 +4370,7 @@
       </c>
       <c r="B42" s="20" t="inlineStr">
         <is>
-          <t>Retrieval Agents</t>
+          <t>Sandbox</t>
         </is>
       </c>
       <c r="C42" s="20" t="inlineStr"/>
@@ -4404,7 +4386,7 @@
       </c>
       <c r="B43" s="20" t="inlineStr">
         <is>
-          <t>Sandbox</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="C43" s="20" t="inlineStr"/>
@@ -4420,7 +4402,7 @@
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Cybersecurity</t>
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr"/>
@@ -4436,13 +4418,29 @@
       </c>
       <c r="B45" s="20" t="inlineStr">
         <is>
-          <t>Cybersecurity</t>
-        </is>
-      </c>
-      <c r="C45" s="20" t="inlineStr"/>
-      <c r="D45" s="20" t="inlineStr"/>
-      <c r="E45" s="20" t="inlineStr"/>
-      <c r="F45" s="20" t="inlineStr"/>
+          <t>FAIR data</t>
+        </is>
+      </c>
+      <c r="C45" s="20" t="inlineStr">
+        <is>
+          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E45" s="20" t="inlineStr">
+        <is>
+          <t>topic_4012</t>
+        </is>
+      </c>
+      <c r="F45" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_4012</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
@@ -4452,29 +4450,13 @@
       </c>
       <c r="B46" s="20" t="inlineStr">
         <is>
-          <t>FAIR data</t>
-        </is>
-      </c>
-      <c r="C46" s="20" t="inlineStr">
-        <is>
-          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="inlineStr">
-        <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E46" s="20" t="inlineStr">
-        <is>
-          <t>topic_4012</t>
-        </is>
-      </c>
-      <c r="F46" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_4012</t>
-        </is>
-      </c>
+          <t>API Integration</t>
+        </is>
+      </c>
+      <c r="C46" s="20" t="inlineStr"/>
+      <c r="D46" s="20" t="inlineStr"/>
+      <c r="E46" s="20" t="inlineStr"/>
+      <c r="F46" s="20" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
@@ -4484,7 +4466,7 @@
       </c>
       <c r="B47" s="20" t="inlineStr">
         <is>
-          <t>API Integration</t>
+          <t>Model Integration</t>
         </is>
       </c>
       <c r="C47" s="20" t="inlineStr"/>
@@ -4500,7 +4482,7 @@
       </c>
       <c r="B48" s="20" t="inlineStr">
         <is>
-          <t>Model Integration</t>
+          <t>Server Integration</t>
         </is>
       </c>
       <c r="C48" s="20" t="inlineStr"/>
@@ -4516,7 +4498,7 @@
       </c>
       <c r="B49" s="20" t="inlineStr">
         <is>
-          <t>Server Integration</t>
+          <t>Server Patterns</t>
         </is>
       </c>
       <c r="C49" s="20" t="inlineStr"/>
@@ -4527,12 +4509,12 @@
     <row r="50">
       <c r="A50" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B50" s="20" t="inlineStr">
         <is>
-          <t>Server Patterns</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr"/>
@@ -4548,7 +4530,7 @@
       </c>
       <c r="B51" s="20" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C51" s="20" t="inlineStr"/>
@@ -4564,13 +4546,29 @@
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="C52" s="20" t="inlineStr"/>
-      <c r="D52" s="20" t="inlineStr"/>
-      <c r="E52" s="20" t="inlineStr"/>
-      <c r="F52" s="20" t="inlineStr"/>
+          <t>Data governance</t>
+        </is>
+      </c>
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>Focuses specifically on the technical protocols, access controls, data-line security, and de-identification standards used to protect the integrity, quality, and privacy of information throughout its lifecycle</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E52" s="20" t="inlineStr">
+        <is>
+          <t>topic_3571</t>
+        </is>
+      </c>
+      <c r="F52" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3571</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="20" t="inlineStr">
@@ -4580,29 +4578,17 @@
       </c>
       <c r="B53" s="20" t="inlineStr">
         <is>
-          <t>Data governance</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="C53" s="20" t="inlineStr">
         <is>
-          <t>Focuses specifically on the technical protocols, access controls, data-line security, and de-identification standards used to protect the integrity, quality, and privacy of information throughout its lifecycle</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="inlineStr">
-        <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E53" s="20" t="inlineStr">
-        <is>
-          <t>topic_3571</t>
-        </is>
-      </c>
-      <c r="F53" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3571</t>
-        </is>
-      </c>
+          <t>The overarching organizational policies, compliance frameworks, and capital allocation strategies that dictate how an enterprise manages its broader IT infrastructure, risk tolerances, and vendor choices</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr"/>
+      <c r="E53" s="20" t="inlineStr"/>
+      <c r="F53" s="20" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="20" t="inlineStr">
@@ -4612,14 +4598,10 @@
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="C54" s="20" t="inlineStr">
-        <is>
-          <t>The overarching organizational policies, compliance frameworks, and capital allocation strategies that dictate how an enterprise manages its broader IT infrastructure, risk tolerances, and vendor choices</t>
-        </is>
-      </c>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr"/>
       <c r="D54" s="20" t="inlineStr"/>
       <c r="E54" s="20" t="inlineStr"/>
       <c r="F54" s="20" t="inlineStr"/>
@@ -4632,10 +4614,14 @@
       </c>
       <c r="B55" s="20" t="inlineStr">
         <is>
-          <t>Implementation</t>
-        </is>
-      </c>
-      <c r="C55" s="20" t="inlineStr"/>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>The tactical, hands-on execution of installing, configuring, provisioning, and launching software or hardware systems within a specific operational environment</t>
+        </is>
+      </c>
       <c r="D55" s="20" t="inlineStr"/>
       <c r="E55" s="20" t="inlineStr"/>
       <c r="F55" s="20" t="inlineStr"/>
@@ -4648,17 +4634,25 @@
       </c>
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t>Deployment</t>
-        </is>
-      </c>
-      <c r="C56" s="20" t="inlineStr">
-        <is>
-          <t>The tactical, hands-on execution of installing, configuring, provisioning, and launching software or hardware systems within a specific operational environment</t>
-        </is>
-      </c>
-      <c r="D56" s="20" t="inlineStr"/>
-      <c r="E56" s="20" t="inlineStr"/>
-      <c r="F56" s="20" t="inlineStr"/>
+          <t>Workflows</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr"/>
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>topic_0769</t>
+        </is>
+      </c>
+      <c r="F56" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_0769</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="20" t="inlineStr">
@@ -4668,25 +4662,13 @@
       </c>
       <c r="B57" s="20" t="inlineStr">
         <is>
-          <t>Workflows</t>
+          <t>Model selection</t>
         </is>
       </c>
       <c r="C57" s="20" t="inlineStr"/>
-      <c r="D57" s="20" t="inlineStr">
-        <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>topic_0769</t>
-        </is>
-      </c>
-      <c r="F57" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_0769</t>
-        </is>
-      </c>
+      <c r="D57" s="20" t="inlineStr"/>
+      <c r="E57" s="20" t="inlineStr"/>
+      <c r="F57" s="20" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="20" t="inlineStr">
@@ -4696,7 +4678,7 @@
       </c>
       <c r="B58" s="20" t="inlineStr">
         <is>
-          <t>Workflow integration</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr"/>
@@ -4712,10 +4694,14 @@
       </c>
       <c r="B59" s="20" t="inlineStr">
         <is>
-          <t>Model selection</t>
-        </is>
-      </c>
-      <c r="C59" s="20" t="inlineStr"/>
+          <t>Architecture Compute</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>Physical node topologies, hardware constraints, VRAM bounds, and localized compute execution profiles.</t>
+        </is>
+      </c>
       <c r="D59" s="20" t="inlineStr"/>
       <c r="E59" s="20" t="inlineStr"/>
       <c r="F59" s="20" t="inlineStr"/>
@@ -4728,10 +4714,14 @@
       </c>
       <c r="B60" s="20" t="inlineStr">
         <is>
-          <t>Evaluation</t>
-        </is>
-      </c>
-      <c r="C60" s="20" t="inlineStr"/>
+          <t>Network Isolation</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>Non-egress boundaries, air-gapped artifact staging, localized cloud VPC containers, and firewalled local registries.</t>
+        </is>
+      </c>
       <c r="D60" s="20" t="inlineStr"/>
       <c r="E60" s="20" t="inlineStr"/>
       <c r="F60" s="20" t="inlineStr"/>
@@ -4744,12 +4734,12 @@
       </c>
       <c r="B61" s="20" t="inlineStr">
         <is>
-          <t>Architecture Compute</t>
+          <t>Infrastructure Security</t>
         </is>
       </c>
       <c r="C61" s="20" t="inlineStr">
         <is>
-          <t>Physical node topologies, hardware constraints, VRAM bounds, and localized compute execution profiles.</t>
+          <t>For on-prem LLM deployments, it captures the security of the compute stack as well as the data pipelines</t>
         </is>
       </c>
       <c r="D61" s="20" t="inlineStr"/>
@@ -4764,12 +4754,12 @@
       </c>
       <c r="B62" s="20" t="inlineStr">
         <is>
-          <t>Network Isolation</t>
+          <t>Self‑hosted AI</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
         <is>
-          <t>Non-egress boundaries, air-gapped artifact staging, localized cloud VPC containers, and firewalled local registries.</t>
+          <t>Self‑hosted, open‑weights models in contrast to API‑based models like OpenAI, Anthropic, or Gemini</t>
         </is>
       </c>
       <c r="D62" s="20" t="inlineStr"/>
@@ -4784,17 +4774,29 @@
       </c>
       <c r="B63" s="20" t="inlineStr">
         <is>
-          <t>Infrastructure Security</t>
+          <t>Data Protection</t>
         </is>
       </c>
       <c r="C63" s="20" t="inlineStr">
         <is>
-          <t>For on-prem LLM deployments, it captures the security of the compute stack as well as the data pipelines</t>
-        </is>
-      </c>
-      <c r="D63" s="20" t="inlineStr"/>
-      <c r="E63" s="20" t="inlineStr"/>
-      <c r="F63" s="20" t="inlineStr"/>
+          <t>Safeguarding sensitive data specifically. Distinct from the broader Security term.</t>
+        </is>
+      </c>
+      <c r="D63" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>topic_4044</t>
+        </is>
+      </c>
+      <c r="F63" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_4044</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="20" t="inlineStr">
@@ -4804,17 +4806,29 @@
       </c>
       <c r="B64" s="20" t="inlineStr">
         <is>
-          <t>Self‑hosted AI</t>
+          <t>FAIR data</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
-          <t>Self‑hosted, open‑weights models in contrast to API‑based models like OpenAI, Anthropic, or Gemini</t>
-        </is>
-      </c>
-      <c r="D64" s="20" t="inlineStr"/>
-      <c r="E64" s="20" t="inlineStr"/>
-      <c r="F64" s="20" t="inlineStr"/>
+          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
+        </is>
+      </c>
+      <c r="D64" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>topic_4012</t>
+        </is>
+      </c>
+      <c r="F64" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_4012</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="20" t="inlineStr">
@@ -4824,14 +4838,10 @@
       </c>
       <c r="B65" s="20" t="inlineStr">
         <is>
-          <t>Data Protection</t>
-        </is>
-      </c>
-      <c r="C65" s="20" t="inlineStr">
-        <is>
-          <t>Safeguarding sensitive data specifically. Distinct from the broader Security term.</t>
-        </is>
-      </c>
+          <t>Data quality management</t>
+        </is>
+      </c>
+      <c r="C65" s="20" t="inlineStr"/>
       <c r="D65" s="20" t="inlineStr">
         <is>
           <t>EDAM</t>
@@ -4839,12 +4849,12 @@
       </c>
       <c r="E65" s="20" t="inlineStr">
         <is>
-          <t>topic_4044</t>
+          <t>topic_3572</t>
         </is>
       </c>
       <c r="F65" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_4044</t>
+          <t>http://edamontology.org/topic_3572</t>
         </is>
       </c>
     </row>
@@ -4856,14 +4866,10 @@
       </c>
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>FAIR data</t>
-        </is>
-      </c>
-      <c r="C66" s="20" t="inlineStr">
-        <is>
-          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
-        </is>
-      </c>
+          <t>Data curation and archival</t>
+        </is>
+      </c>
+      <c r="C66" s="20" t="inlineStr"/>
       <c r="D66" s="20" t="inlineStr">
         <is>
           <t>EDAM</t>
@@ -4871,12 +4877,12 @@
       </c>
       <c r="E66" s="20" t="inlineStr">
         <is>
-          <t>topic_4012</t>
+          <t>topic_0219</t>
         </is>
       </c>
       <c r="F66" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_4012</t>
+          <t>http://edamontology.org/topic_0219</t>
         </is>
       </c>
     </row>
@@ -4888,7 +4894,7 @@
       </c>
       <c r="B67" s="20" t="inlineStr">
         <is>
-          <t>Data quality management</t>
+          <t>Data integration and warehousing</t>
         </is>
       </c>
       <c r="C67" s="20" t="inlineStr"/>
@@ -4899,12 +4905,12 @@
       </c>
       <c r="E67" s="20" t="inlineStr">
         <is>
-          <t>topic_3572</t>
+          <t>topic_3366</t>
         </is>
       </c>
       <c r="F67" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_3572</t>
+          <t>http://edamontology.org/topic_3366</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4922,7 @@
       </c>
       <c r="B68" s="20" t="inlineStr">
         <is>
-          <t>Data curation and archival</t>
+          <t>Data architecture, analysis and design</t>
         </is>
       </c>
       <c r="C68" s="20" t="inlineStr"/>
@@ -4927,12 +4933,12 @@
       </c>
       <c r="E68" s="20" t="inlineStr">
         <is>
-          <t>topic_0219</t>
+          <t>topic_3365</t>
         </is>
       </c>
       <c r="F68" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_0219</t>
+          <t>http://edamontology.org/topic_3365</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4950,7 @@
       </c>
       <c r="B69" s="20" t="inlineStr">
         <is>
-          <t>Data integration and warehousing</t>
+          <t>Data identity and mapping</t>
         </is>
       </c>
       <c r="C69" s="20" t="inlineStr"/>
@@ -4955,12 +4961,12 @@
       </c>
       <c r="E69" s="20" t="inlineStr">
         <is>
-          <t>topic_3366</t>
+          <t>topic_3345</t>
         </is>
       </c>
       <c r="F69" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_3366</t>
+          <t>http://edamontology.org/topic_3345</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4978,7 @@
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>Data architecture, analysis and design</t>
+          <t>Data rescue</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr"/>
@@ -4983,12 +4989,12 @@
       </c>
       <c r="E70" s="20" t="inlineStr">
         <is>
-          <t>topic_3365</t>
+          <t>topic_4011</t>
         </is>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_3365</t>
+          <t>http://edamontology.org/topic_4011</t>
         </is>
       </c>
     </row>
@@ -5000,25 +5006,21 @@
       </c>
       <c r="B71" s="20" t="inlineStr">
         <is>
-          <t>Data identity and mapping</t>
-        </is>
-      </c>
-      <c r="C71" s="20" t="inlineStr"/>
+          <t>Valid and Reliable</t>
+        </is>
+      </c>
+      <c r="C71" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D71" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E71" s="20" t="inlineStr">
-        <is>
-          <t>topic_3345</t>
-        </is>
-      </c>
-      <c r="F71" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3345</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E71" s="20" t="inlineStr"/>
+      <c r="F71" s="20" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="20" t="inlineStr">
@@ -5028,25 +5030,21 @@
       </c>
       <c r="B72" s="20" t="inlineStr">
         <is>
-          <t>Data rescue</t>
-        </is>
-      </c>
-      <c r="C72" s="20" t="inlineStr"/>
+          <t>Safe</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D72" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E72" s="20" t="inlineStr">
-        <is>
-          <t>topic_4011</t>
-        </is>
-      </c>
-      <c r="F72" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_4011</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E72" s="20" t="inlineStr"/>
+      <c r="F72" s="20" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="20" t="inlineStr">
@@ -5056,7 +5054,7 @@
       </c>
       <c r="B73" s="20" t="inlineStr">
         <is>
-          <t>Valid and Reliable</t>
+          <t>Secure and Resilient</t>
         </is>
       </c>
       <c r="C73" s="20" t="inlineStr">
@@ -5080,7 +5078,7 @@
       </c>
       <c r="B74" s="20" t="inlineStr">
         <is>
-          <t>Safe</t>
+          <t>Accountable and Transparent</t>
         </is>
       </c>
       <c r="C74" s="20" t="inlineStr">
@@ -5104,7 +5102,7 @@
       </c>
       <c r="B75" s="20" t="inlineStr">
         <is>
-          <t>Secure and Resilient</t>
+          <t>Explainable and Interpretable</t>
         </is>
       </c>
       <c r="C75" s="20" t="inlineStr">
@@ -5128,7 +5126,7 @@
       </c>
       <c r="B76" s="20" t="inlineStr">
         <is>
-          <t>Accountable and Transparent</t>
+          <t>Privacy-Enhanced</t>
         </is>
       </c>
       <c r="C76" s="20" t="inlineStr">
@@ -5152,12 +5150,12 @@
       </c>
       <c r="B77" s="20" t="inlineStr">
         <is>
-          <t>Explainable and Interpretable</t>
+          <t>Fair (harmful bias managed)</t>
         </is>
       </c>
       <c r="C77" s="20" t="inlineStr">
         <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+          <t>NIST AI RMF trustworthy-AI characteristic: algorithmic non-discrimination. NOT the same as 'FAIR data'.</t>
         </is>
       </c>
       <c r="D77" s="20" t="inlineStr">
@@ -5171,48 +5169,32 @@
     <row r="78">
       <c r="A78" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B78" s="20" t="inlineStr">
         <is>
-          <t>Privacy-Enhanced</t>
-        </is>
-      </c>
-      <c r="C78" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D78" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr"/>
+      <c r="D78" s="20" t="inlineStr"/>
       <c r="E78" s="20" t="inlineStr"/>
       <c r="F78" s="20" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B79" s="20" t="inlineStr">
         <is>
-          <t>Fair (harmful bias managed)</t>
-        </is>
-      </c>
-      <c r="C79" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic: algorithmic non-discrimination. NOT the same as 'FAIR data'.</t>
-        </is>
-      </c>
-      <c r="D79" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr"/>
+      <c r="D79" s="20" t="inlineStr"/>
       <c r="E79" s="20" t="inlineStr"/>
       <c r="F79" s="20" t="inlineStr"/>
     </row>
@@ -5224,7 +5206,7 @@
       </c>
       <c r="B80" s="20" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Mature</t>
         </is>
       </c>
       <c r="C80" s="20" t="inlineStr"/>
@@ -5240,45 +5222,13 @@
       </c>
       <c r="B81" s="20" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Deprecated</t>
         </is>
       </c>
       <c r="C81" s="20" t="inlineStr"/>
       <c r="D81" s="20" t="inlineStr"/>
       <c r="E81" s="20" t="inlineStr"/>
       <c r="F81" s="20" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B82" s="20" t="inlineStr">
-        <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="C82" s="20" t="inlineStr"/>
-      <c r="D82" s="20" t="inlineStr"/>
-      <c r="E82" s="20" t="inlineStr"/>
-      <c r="F82" s="20" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B83" s="20" t="inlineStr">
-        <is>
-          <t>Deprecated</t>
-        </is>
-      </c>
-      <c r="C83" s="20" t="inlineStr"/>
-      <c r="D83" s="20" t="inlineStr"/>
-      <c r="E83" s="20" t="inlineStr"/>
-      <c r="F83" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add ACM-CCS as a standard, map 7 terms with genuine matches
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -4166,9 +4166,21 @@
         </is>
       </c>
       <c r="C29" s="20" t="inlineStr"/>
-      <c r="D29" s="20" t="inlineStr"/>
-      <c r="E29" s="20" t="inlineStr"/>
-      <c r="F29" s="20" t="inlineStr"/>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E29" s="20" t="inlineStr">
+        <is>
+          <t>Software and its engineering~Software verification and validation~Software testing and debugging</t>
+        </is>
+      </c>
+      <c r="F29" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
@@ -4342,9 +4354,21 @@
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr"/>
-      <c r="D40" s="20" t="inlineStr"/>
-      <c r="E40" s="20" t="inlineStr"/>
-      <c r="F40" s="20" t="inlineStr"/>
+      <c r="D40" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E40" s="20" t="inlineStr">
+        <is>
+          <t>Information systems~Information retrieval</t>
+        </is>
+      </c>
+      <c r="F40" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="20" t="inlineStr">
@@ -4358,9 +4382,21 @@
         </is>
       </c>
       <c r="C41" s="20" t="inlineStr"/>
-      <c r="D41" s="20" t="inlineStr"/>
-      <c r="E41" s="20" t="inlineStr"/>
-      <c r="F41" s="20" t="inlineStr"/>
+      <c r="D41" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E41" s="20" t="inlineStr">
+        <is>
+          <t>Information systems~Information retrieval</t>
+        </is>
+      </c>
+      <c r="F41" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="20" t="inlineStr">
@@ -4406,9 +4442,21 @@
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr"/>
-      <c r="D44" s="20" t="inlineStr"/>
-      <c r="E44" s="20" t="inlineStr"/>
-      <c r="F44" s="20" t="inlineStr"/>
+      <c r="D44" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E44" s="20" t="inlineStr">
+        <is>
+          <t>Security and privacy</t>
+        </is>
+      </c>
+      <c r="F44" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
@@ -4518,9 +4566,21 @@
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr"/>
-      <c r="D50" s="20" t="inlineStr"/>
-      <c r="E50" s="20" t="inlineStr"/>
-      <c r="F50" s="20" t="inlineStr"/>
+      <c r="D50" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E50" s="20" t="inlineStr">
+        <is>
+          <t>Computer systems organization~Architectures</t>
+        </is>
+      </c>
+      <c r="F50" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="20" t="inlineStr">
@@ -4534,9 +4594,21 @@
         </is>
       </c>
       <c r="C51" s="20" t="inlineStr"/>
-      <c r="D51" s="20" t="inlineStr"/>
-      <c r="E51" s="20" t="inlineStr"/>
-      <c r="F51" s="20" t="inlineStr"/>
+      <c r="D51" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>Security and privacy</t>
+        </is>
+      </c>
+      <c r="F51" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="20" t="inlineStr">
@@ -4682,9 +4754,21 @@
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr"/>
-      <c r="D58" s="20" t="inlineStr"/>
-      <c r="E58" s="20" t="inlineStr"/>
-      <c r="F58" s="20" t="inlineStr"/>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>Software and its engineering~Software verification and validation~Software testing and debugging</t>
+        </is>
+      </c>
+      <c r="F58" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="20" t="inlineStr">
@@ -5241,7 +5325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -5332,6 +5416,33 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ACM Computing Classification System (CCS 2012)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cited by category path text (e.g. "Computer systems organization~Architectures"), not a numeric ID a human needs to look up -- confirmed against real paper citations. General computing/software-engineering taxonomy, not agentic-AI-specific -- predates MCP, agent frameworks, and tool-calling entirely, so it backs general CS terms (Architecture, Security, Evaluation, Retrieval) but not agent-specific ones (MCP, Hooks, Skills, Orchestration, ...). Path spellings below are from established domain knowledge, not a live verified fetch (dl.acm.org blocked automated access) -- worth spot-checking in a browser before treating as fully authoritative.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename Architecture Compute to Compute Infrastructure; map Implementation and Deployment
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -1987,7 +1987,7 @@
       </c>
       <c r="J26" s="16" t="inlineStr">
         <is>
-          <t>Self‑hosted AI; Architecture Compute; Implementation; Network Isolation; Infrastructure Security</t>
+          <t>Self‑hosted AI; Compute Infrastructure; Implementation; Network Isolation; Infrastructure Security</t>
         </is>
       </c>
       <c r="K26" s="16" t="inlineStr">
@@ -4674,9 +4674,21 @@
         </is>
       </c>
       <c r="C54" s="20" t="inlineStr"/>
-      <c r="D54" s="20" t="inlineStr"/>
-      <c r="E54" s="20" t="inlineStr"/>
-      <c r="F54" s="20" t="inlineStr"/>
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>Software and its engineering~Software creation and management</t>
+        </is>
+      </c>
+      <c r="F54" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="20" t="inlineStr">
@@ -4694,9 +4706,21 @@
           <t>The tactical, hands-on execution of installing, configuring, provisioning, and launching software or hardware systems within a specific operational environment</t>
         </is>
       </c>
-      <c r="D55" s="20" t="inlineStr"/>
-      <c r="E55" s="20" t="inlineStr"/>
-      <c r="F55" s="20" t="inlineStr"/>
+      <c r="D55" s="20" t="inlineStr">
+        <is>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>AI lifecycle stage: Deploy</t>
+        </is>
+      </c>
+      <c r="F55" s="20" t="inlineStr">
+        <is>
+          <t>https://nvlpubs.nist.gov/nistpubs/ai/NIST.AI.100-1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="20" t="inlineStr">
@@ -4778,7 +4802,7 @@
       </c>
       <c r="B59" s="20" t="inlineStr">
         <is>
-          <t>Architecture Compute</t>
+          <t>Compute Infrastructure</t>
         </is>
       </c>
       <c r="C59" s="20" t="inlineStr">
@@ -5412,32 +5436,32 @@
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
-          <t>Optional secondary axis: the seven trustworthy-AI characteristics. Document-based, so individual characteristics have no per-term URIs. WARNING: NIST's 'Fair (harmful bias managed)' concerns algorithmic non-discrimination and is UNRELATED to EDAM's 'FAIR data' (Findable / Accessible / Interoperable / Reusable data principles) despite sharing the word - do not conflate the two.</t>
+          <t>Optional secondary axis: the seven trustworthy-AI characteristics. Document-based, so individual characteristics have no per-term URIs. WARNING: NIST's 'Fair (harmful bias managed)' concerns algorithmic non-discrimination and is UNRELATED to EDAM's 'FAIR data' (Findable / Accessible / Interoperable / Reusable data principles) despite sharing the word - do not conflate the two. Also defines an AI lifecycle with named stages (plan, collect/process, build, verify, deploy, operate) -- cited here as e.g. "AI lifecycle stage: Deploy", distinct from the seven trustworthy-AI characteristics.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>ACM-CCS</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>ACM Computing Classification System (CCS 2012)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>2012</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>https://dl.acm.org/ccs</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>Cited by category path text (e.g. "Computer systems organization~Architectures"), not a numeric ID a human needs to look up -- confirmed against real paper citations. General computing/software-engineering taxonomy, not agentic-AI-specific -- predates MCP, agent frameworks, and tool-calling entirely, so it backs general CS terms (Architecture, Security, Evaluation, Retrieval) but not agent-specific ones (MCP, Hooks, Skills, Orchestration, ...). Path spellings below are from established domain knowledge, not a live verified fetch (dl.acm.org blocked automated access) -- worth spot-checking in a browser before treating as fully authoritative.</t>
         </is>

</xml_diff>

<commit_message>
Add Schema.org as a standard, map 13 Resource Type terms
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -3718,9 +3718,21 @@
         </is>
       </c>
       <c r="C2" s="20" t="inlineStr"/>
-      <c r="D2" s="20" t="inlineStr"/>
-      <c r="E2" s="20" t="inlineStr"/>
-      <c r="F2" s="20" t="inlineStr"/>
+      <c r="D2" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>schema:TechArticle</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/TechArticle</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -3734,9 +3746,21 @@
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr"/>
-      <c r="D3" s="20" t="inlineStr"/>
-      <c r="E3" s="20" t="inlineStr"/>
-      <c r="F3" s="20" t="inlineStr"/>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>schema:APIReference</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/APIReference</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
@@ -3750,9 +3774,21 @@
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr"/>
-      <c r="D4" s="20" t="inlineStr"/>
-      <c r="E4" s="20" t="inlineStr"/>
-      <c r="F4" s="20" t="inlineStr"/>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>schema:TechArticle</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/TechArticle</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
@@ -3770,9 +3806,21 @@
           <t>Vendor or organization technical whitepaper.</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr"/>
-      <c r="E5" s="20" t="inlineStr"/>
-      <c r="F5" s="20" t="inlineStr"/>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>schema:TechArticle</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/TechArticle</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
@@ -3790,9 +3838,21 @@
           <t>Peer-reviewed publication or preprint. Distinct from a vendor Whitepaper.</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr"/>
-      <c r="E6" s="20" t="inlineStr"/>
-      <c r="F6" s="20" t="inlineStr"/>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>schema:ScholarlyArticle</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/ScholarlyArticle</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
@@ -3806,9 +3866,21 @@
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr"/>
-      <c r="D7" s="20" t="inlineStr"/>
-      <c r="E7" s="20" t="inlineStr"/>
-      <c r="F7" s="20" t="inlineStr"/>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>schema:TechArticle</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/TechArticle</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
@@ -3822,9 +3894,21 @@
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr"/>
-      <c r="D8" s="20" t="inlineStr"/>
-      <c r="E8" s="20" t="inlineStr"/>
-      <c r="F8" s="20" t="inlineStr"/>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>schema:TechArticle</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/TechArticle</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
@@ -3838,9 +3922,21 @@
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr"/>
-      <c r="D9" s="20" t="inlineStr"/>
-      <c r="E9" s="20" t="inlineStr"/>
-      <c r="F9" s="20" t="inlineStr"/>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>schema:TechArticle</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/TechArticle</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
@@ -3918,9 +4014,21 @@
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr"/>
-      <c r="D14" s="20" t="inlineStr"/>
-      <c r="E14" s="20" t="inlineStr"/>
-      <c r="F14" s="20" t="inlineStr"/>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>schema:SoftwareSourceCode</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/SoftwareSourceCode</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
@@ -3938,9 +4046,21 @@
           <t>A curated collection of benchmarks or comparison studies.</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr"/>
-      <c r="E15" s="20" t="inlineStr"/>
-      <c r="F15" s="20" t="inlineStr"/>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>schema:Dataset</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/Dataset</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
@@ -3970,9 +4090,21 @@
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr"/>
-      <c r="D17" s="20" t="inlineStr"/>
-      <c r="E17" s="20" t="inlineStr"/>
-      <c r="F17" s="20" t="inlineStr"/>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>schema:BlogPosting</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/BlogPosting</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
@@ -3986,9 +4118,21 @@
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr"/>
-      <c r="D18" s="20" t="inlineStr"/>
-      <c r="E18" s="20" t="inlineStr"/>
-      <c r="F18" s="20" t="inlineStr"/>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>schema:SoftwareSourceCode</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/SoftwareSourceCode</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="inlineStr">
@@ -4002,9 +4146,21 @@
         </is>
       </c>
       <c r="C19" s="20" t="inlineStr"/>
-      <c r="D19" s="20" t="inlineStr"/>
-      <c r="E19" s="20" t="inlineStr"/>
-      <c r="F19" s="20" t="inlineStr"/>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>schema:TechArticle</t>
+        </is>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>https://schema.org/TechArticle</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
@@ -5349,7 +5505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -5467,6 +5623,33 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Schema.org</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Schema.org (CreativeWork hierarchy)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://schema.org/CreativeWork</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Universal web-metadata vocabulary. Exact-type matches applied directly (e.g. APIReference, BlogPosting, ScholarlyArticle, SoftwareSourceCode, Dataset). For highly specific AI-radar terms with no exact schema.org type, the broader parent type is applied instead (e.g. several terms map to TechArticle) -- this is schema.org's own intended usage pattern (broad type + a custom category property), not a forced fit, but it means several distinct Resource Type terms intentionally share one Ontology ID here, unlike EDAM/ACM-CCS/NIST-AI-RMF where each backed term has its own distinct match.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove unused Resource Type vocabulary terms
Architecture Pattern, Blog Post, Example Repo, and Tutorial were never
used by any row and are dropped from the Vocabulary tab.
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -3663,7 +3663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="17" min="1" max="1"/>
@@ -4065,12 +4065,12 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Resource Type</t>
+          <t>Agentic Features Covered</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Tutorial</t>
+          <t>Hooks</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr"/>
@@ -4081,86 +4081,54 @@
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Resource Type</t>
+          <t>Agentic Features Covered</t>
         </is>
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Skills</t>
         </is>
       </c>
       <c r="C17" s="20" t="inlineStr"/>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>Schema.org</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>schema:BlogPosting</t>
-        </is>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>https://schema.org/BlogPosting</t>
-        </is>
-      </c>
+      <c r="D17" s="20" t="inlineStr"/>
+      <c r="E17" s="20" t="inlineStr"/>
+      <c r="F17" s="20" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>Resource Type</t>
+          <t>Agentic Features Covered</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Example Repo</t>
-        </is>
-      </c>
-      <c r="C18" s="20" t="inlineStr"/>
-      <c r="D18" s="20" t="inlineStr">
-        <is>
-          <t>Schema.org</t>
-        </is>
-      </c>
-      <c r="E18" s="20" t="inlineStr">
-        <is>
-          <t>schema:SoftwareSourceCode</t>
-        </is>
-      </c>
-      <c r="F18" s="20" t="inlineStr">
-        <is>
-          <t>https://schema.org/SoftwareSourceCode</t>
-        </is>
-      </c>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Model Context Protocol.</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr"/>
+      <c r="E18" s="20" t="inlineStr"/>
+      <c r="F18" s="20" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>Resource Type</t>
+          <t>Agentic Features Covered</t>
         </is>
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>Architecture Pattern</t>
+          <t>Agent frameworks</t>
         </is>
       </c>
       <c r="C19" s="20" t="inlineStr"/>
-      <c r="D19" s="20" t="inlineStr">
-        <is>
-          <t>Schema.org</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="inlineStr">
-        <is>
-          <t>schema:TechArticle</t>
-        </is>
-      </c>
-      <c r="F19" s="20" t="inlineStr">
-        <is>
-          <t>https://schema.org/TechArticle</t>
-        </is>
-      </c>
+      <c r="D19" s="20" t="inlineStr"/>
+      <c r="E19" s="20" t="inlineStr"/>
+      <c r="F19" s="20" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
@@ -4170,7 +4138,7 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Hooks</t>
+          <t>Agent Patterns</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr"/>
@@ -4186,7 +4154,7 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>Skills</t>
+          <t>Multi-Agent Patterns</t>
         </is>
       </c>
       <c r="C21" s="20" t="inlineStr"/>
@@ -4202,14 +4170,10 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>MCP</t>
-        </is>
-      </c>
-      <c r="C22" s="20" t="inlineStr">
-        <is>
-          <t>Model Context Protocol.</t>
-        </is>
-      </c>
+          <t>Context window management</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr"/>
       <c r="D22" s="20" t="inlineStr"/>
       <c r="E22" s="20" t="inlineStr"/>
       <c r="F22" s="20" t="inlineStr"/>
@@ -4222,7 +4186,7 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Agent frameworks</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="C23" s="20" t="inlineStr"/>
@@ -4238,7 +4202,7 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Agent Patterns</t>
+          <t>Safety / guardrails</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr"/>
@@ -4254,13 +4218,25 @@
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>Multi-Agent Patterns</t>
+          <t>Evaluation / testing</t>
         </is>
       </c>
       <c r="C25" s="20" t="inlineStr"/>
-      <c r="D25" s="20" t="inlineStr"/>
-      <c r="E25" s="20" t="inlineStr"/>
-      <c r="F25" s="20" t="inlineStr"/>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>Software and its engineering~Software verification and validation~Software testing and debugging</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="20" t="inlineStr">
@@ -4270,7 +4246,7 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Context window management</t>
+          <t>Risk Controls</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr"/>
@@ -4286,7 +4262,7 @@
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>Deployment patterns</t>
+          <t>Safe Tool Use</t>
         </is>
       </c>
       <c r="C27" s="20" t="inlineStr"/>
@@ -4302,7 +4278,7 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Safety / guardrails</t>
+          <t>Tools</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr"/>
@@ -4318,25 +4294,13 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>Evaluation / testing</t>
+          <t>Tool-Ready Endpoints</t>
         </is>
       </c>
       <c r="C29" s="20" t="inlineStr"/>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>ACM-CCS</t>
-        </is>
-      </c>
-      <c r="E29" s="20" t="inlineStr">
-        <is>
-          <t>Software and its engineering~Software verification and validation~Software testing and debugging</t>
-        </is>
-      </c>
-      <c r="F29" s="20" t="inlineStr">
-        <is>
-          <t>https://dl.acm.org/ccs</t>
-        </is>
-      </c>
+      <c r="D29" s="20" t="inlineStr"/>
+      <c r="E29" s="20" t="inlineStr"/>
+      <c r="F29" s="20" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="20" t="inlineStr">
@@ -4346,7 +4310,7 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>Risk Controls</t>
+          <t>Coding Agents</t>
         </is>
       </c>
       <c r="C30" s="20" t="inlineStr"/>
@@ -4362,7 +4326,7 @@
       </c>
       <c r="B31" s="20" t="inlineStr">
         <is>
-          <t>Safe Tool Use</t>
+          <t>Notebook Agents</t>
         </is>
       </c>
       <c r="C31" s="20" t="inlineStr"/>
@@ -4378,7 +4342,7 @@
       </c>
       <c r="B32" s="20" t="inlineStr">
         <is>
-          <t>Tools</t>
+          <t>Workflow Agents</t>
         </is>
       </c>
       <c r="C32" s="20" t="inlineStr"/>
@@ -4394,7 +4358,7 @@
       </c>
       <c r="B33" s="20" t="inlineStr">
         <is>
-          <t>Tool-Ready Endpoints</t>
+          <t>Workflow Automation</t>
         </is>
       </c>
       <c r="C33" s="20" t="inlineStr"/>
@@ -4410,7 +4374,7 @@
       </c>
       <c r="B34" s="20" t="inlineStr">
         <is>
-          <t>Coding Agents</t>
+          <t>Orchestration</t>
         </is>
       </c>
       <c r="C34" s="20" t="inlineStr"/>
@@ -4426,7 +4390,7 @@
       </c>
       <c r="B35" s="20" t="inlineStr">
         <is>
-          <t>Notebook Agents</t>
+          <t>Triggers</t>
         </is>
       </c>
       <c r="C35" s="20" t="inlineStr"/>
@@ -4442,13 +4406,25 @@
       </c>
       <c r="B36" s="20" t="inlineStr">
         <is>
-          <t>Workflow Agents</t>
+          <t>Retrieval</t>
         </is>
       </c>
       <c r="C36" s="20" t="inlineStr"/>
-      <c r="D36" s="20" t="inlineStr"/>
-      <c r="E36" s="20" t="inlineStr"/>
-      <c r="F36" s="20" t="inlineStr"/>
+      <c r="D36" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E36" s="20" t="inlineStr">
+        <is>
+          <t>Information systems~Information retrieval</t>
+        </is>
+      </c>
+      <c r="F36" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="20" t="inlineStr">
@@ -4458,13 +4434,25 @@
       </c>
       <c r="B37" s="20" t="inlineStr">
         <is>
-          <t>Workflow Automation</t>
+          <t>Retrieval Agents</t>
         </is>
       </c>
       <c r="C37" s="20" t="inlineStr"/>
-      <c r="D37" s="20" t="inlineStr"/>
-      <c r="E37" s="20" t="inlineStr"/>
-      <c r="F37" s="20" t="inlineStr"/>
+      <c r="D37" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E37" s="20" t="inlineStr">
+        <is>
+          <t>Information systems~Information retrieval</t>
+        </is>
+      </c>
+      <c r="F37" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="20" t="inlineStr">
@@ -4474,7 +4462,7 @@
       </c>
       <c r="B38" s="20" t="inlineStr">
         <is>
-          <t>Orchestration</t>
+          <t>Sandbox</t>
         </is>
       </c>
       <c r="C38" s="20" t="inlineStr"/>
@@ -4490,7 +4478,7 @@
       </c>
       <c r="B39" s="20" t="inlineStr">
         <is>
-          <t>Triggers</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="C39" s="20" t="inlineStr"/>
@@ -4506,7 +4494,7 @@
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>Retrieval</t>
+          <t>Cybersecurity</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr"/>
@@ -4517,7 +4505,7 @@
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t>Information systems~Information retrieval</t>
+          <t>Security and privacy</t>
         </is>
       </c>
       <c r="F40" s="20" t="inlineStr">
@@ -4534,23 +4522,27 @@
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
-          <t>Retrieval Agents</t>
-        </is>
-      </c>
-      <c r="C41" s="20" t="inlineStr"/>
+          <t>FAIR data</t>
+        </is>
+      </c>
+      <c r="C41" s="20" t="inlineStr">
+        <is>
+          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
+        </is>
+      </c>
       <c r="D41" s="20" t="inlineStr">
         <is>
-          <t>ACM-CCS</t>
+          <t>EDAM</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Information systems~Information retrieval</t>
+          <t>topic_4012</t>
         </is>
       </c>
       <c r="F41" s="20" t="inlineStr">
         <is>
-          <t>https://dl.acm.org/ccs</t>
+          <t>http://edamontology.org/topic_4012</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4554,7 @@
       </c>
       <c r="B42" s="20" t="inlineStr">
         <is>
-          <t>Sandbox</t>
+          <t>API Integration</t>
         </is>
       </c>
       <c r="C42" s="20" t="inlineStr"/>
@@ -4578,7 +4570,7 @@
       </c>
       <c r="B43" s="20" t="inlineStr">
         <is>
-          <t>Governance</t>
+          <t>Model Integration</t>
         </is>
       </c>
       <c r="C43" s="20" t="inlineStr"/>
@@ -4594,25 +4586,13 @@
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>Cybersecurity</t>
+          <t>Server Integration</t>
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr"/>
-      <c r="D44" s="20" t="inlineStr">
-        <is>
-          <t>ACM-CCS</t>
-        </is>
-      </c>
-      <c r="E44" s="20" t="inlineStr">
-        <is>
-          <t>Security and privacy</t>
-        </is>
-      </c>
-      <c r="F44" s="20" t="inlineStr">
-        <is>
-          <t>https://dl.acm.org/ccs</t>
-        </is>
-      </c>
+      <c r="D44" s="20" t="inlineStr"/>
+      <c r="E44" s="20" t="inlineStr"/>
+      <c r="F44" s="20" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="20" t="inlineStr">
@@ -4622,90 +4602,118 @@
       </c>
       <c r="B45" s="20" t="inlineStr">
         <is>
-          <t>FAIR data</t>
-        </is>
-      </c>
-      <c r="C45" s="20" t="inlineStr">
-        <is>
-          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
-        </is>
-      </c>
-      <c r="D45" s="20" t="inlineStr">
-        <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E45" s="20" t="inlineStr">
-        <is>
-          <t>topic_4012</t>
-        </is>
-      </c>
-      <c r="F45" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_4012</t>
-        </is>
-      </c>
+          <t>Server Patterns</t>
+        </is>
+      </c>
+      <c r="C45" s="20" t="inlineStr"/>
+      <c r="D45" s="20" t="inlineStr"/>
+      <c r="E45" s="20" t="inlineStr"/>
+      <c r="F45" s="20" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B46" s="20" t="inlineStr">
         <is>
-          <t>API Integration</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="C46" s="20" t="inlineStr"/>
-      <c r="D46" s="20" t="inlineStr"/>
-      <c r="E46" s="20" t="inlineStr"/>
-      <c r="F46" s="20" t="inlineStr"/>
+      <c r="D46" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E46" s="20" t="inlineStr">
+        <is>
+          <t>Computer systems organization~Architectures</t>
+        </is>
+      </c>
+      <c r="F46" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B47" s="20" t="inlineStr">
         <is>
-          <t>Model Integration</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C47" s="20" t="inlineStr"/>
-      <c r="D47" s="20" t="inlineStr"/>
-      <c r="E47" s="20" t="inlineStr"/>
-      <c r="F47" s="20" t="inlineStr"/>
+      <c r="D47" s="20" t="inlineStr">
+        <is>
+          <t>ACM-CCS</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Security and privacy</t>
+        </is>
+      </c>
+      <c r="F47" s="20" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/ccs</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B48" s="20" t="inlineStr">
         <is>
-          <t>Server Integration</t>
-        </is>
-      </c>
-      <c r="C48" s="20" t="inlineStr"/>
-      <c r="D48" s="20" t="inlineStr"/>
-      <c r="E48" s="20" t="inlineStr"/>
-      <c r="F48" s="20" t="inlineStr"/>
+          <t>Data governance</t>
+        </is>
+      </c>
+      <c r="C48" s="20" t="inlineStr">
+        <is>
+          <t>Focuses specifically on the technical protocols, access controls, data-line security, and de-identification standards used to protect the integrity, quality, and privacy of information throughout its lifecycle</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E48" s="20" t="inlineStr">
+        <is>
+          <t>topic_3571</t>
+        </is>
+      </c>
+      <c r="F48" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3571</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="20" t="inlineStr">
         <is>
-          <t>Agentic Features Covered</t>
+          <t>Topic Focus</t>
         </is>
       </c>
       <c r="B49" s="20" t="inlineStr">
         <is>
-          <t>Server Patterns</t>
-        </is>
-      </c>
-      <c r="C49" s="20" t="inlineStr"/>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="C49" s="20" t="inlineStr">
+        <is>
+          <t>The overarching organizational policies, compliance frameworks, and capital allocation strategies that dictate how an enterprise manages its broader IT infrastructure, risk tolerances, and vendor choices</t>
+        </is>
+      </c>
       <c r="D49" s="20" t="inlineStr"/>
       <c r="E49" s="20" t="inlineStr"/>
       <c r="F49" s="20" t="inlineStr"/>
@@ -4718,7 +4726,7 @@
       </c>
       <c r="B50" s="20" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>Implementation</t>
         </is>
       </c>
       <c r="C50" s="20" t="inlineStr"/>
@@ -4729,7 +4737,7 @@
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>Computer systems organization~Architectures</t>
+          <t>Software and its engineering~Software creation and management</t>
         </is>
       </c>
       <c r="F50" s="20" t="inlineStr">
@@ -4746,23 +4754,27 @@
       </c>
       <c r="B51" s="20" t="inlineStr">
         <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="C51" s="20" t="inlineStr"/>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C51" s="20" t="inlineStr">
+        <is>
+          <t>The tactical, hands-on execution of installing, configuring, provisioning, and launching software or hardware systems within a specific operational environment</t>
+        </is>
+      </c>
       <c r="D51" s="20" t="inlineStr">
         <is>
-          <t>ACM-CCS</t>
+          <t>NIST-AI-RMF</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Security and privacy</t>
+          <t>AI lifecycle stage: Deploy</t>
         </is>
       </c>
       <c r="F51" s="20" t="inlineStr">
         <is>
-          <t>https://dl.acm.org/ccs</t>
+          <t>https://nvlpubs.nist.gov/nistpubs/ai/NIST.AI.100-1.pdf</t>
         </is>
       </c>
     </row>
@@ -4774,14 +4786,10 @@
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
-          <t>Data governance</t>
-        </is>
-      </c>
-      <c r="C52" s="20" t="inlineStr">
-        <is>
-          <t>Focuses specifically on the technical protocols, access controls, data-line security, and de-identification standards used to protect the integrity, quality, and privacy of information throughout its lifecycle</t>
-        </is>
-      </c>
+          <t>Workflows</t>
+        </is>
+      </c>
+      <c r="C52" s="20" t="inlineStr"/>
       <c r="D52" s="20" t="inlineStr">
         <is>
           <t>EDAM</t>
@@ -4789,12 +4797,12 @@
       </c>
       <c r="E52" s="20" t="inlineStr">
         <is>
-          <t>topic_3571</t>
+          <t>topic_0769</t>
         </is>
       </c>
       <c r="F52" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_3571</t>
+          <t>http://edamontology.org/topic_0769</t>
         </is>
       </c>
     </row>
@@ -4806,14 +4814,10 @@
       </c>
       <c r="B53" s="20" t="inlineStr">
         <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="C53" s="20" t="inlineStr">
-        <is>
-          <t>The overarching organizational policies, compliance frameworks, and capital allocation strategies that dictate how an enterprise manages its broader IT infrastructure, risk tolerances, and vendor choices</t>
-        </is>
-      </c>
+          <t>Model selection</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr"/>
       <c r="D53" s="20" t="inlineStr"/>
       <c r="E53" s="20" t="inlineStr"/>
       <c r="F53" s="20" t="inlineStr"/>
@@ -4826,7 +4830,7 @@
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
-          <t>Implementation</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="C54" s="20" t="inlineStr"/>
@@ -4837,7 +4841,7 @@
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
-          <t>Software and its engineering~Software creation and management</t>
+          <t>Software and its engineering~Software verification and validation~Software testing and debugging</t>
         </is>
       </c>
       <c r="F54" s="20" t="inlineStr">
@@ -4854,29 +4858,17 @@
       </c>
       <c r="B55" s="20" t="inlineStr">
         <is>
-          <t>Deployment</t>
+          <t>Compute Infrastructure</t>
         </is>
       </c>
       <c r="C55" s="20" t="inlineStr">
         <is>
-          <t>The tactical, hands-on execution of installing, configuring, provisioning, and launching software or hardware systems within a specific operational environment</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
-      <c r="E55" s="20" t="inlineStr">
-        <is>
-          <t>AI lifecycle stage: Deploy</t>
-        </is>
-      </c>
-      <c r="F55" s="20" t="inlineStr">
-        <is>
-          <t>https://nvlpubs.nist.gov/nistpubs/ai/NIST.AI.100-1.pdf</t>
-        </is>
-      </c>
+          <t>Physical node topologies, hardware constraints, VRAM bounds, and localized compute execution profiles.</t>
+        </is>
+      </c>
+      <c r="D55" s="20" t="inlineStr"/>
+      <c r="E55" s="20" t="inlineStr"/>
+      <c r="F55" s="20" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="20" t="inlineStr">
@@ -4886,25 +4878,17 @@
       </c>
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t>Workflows</t>
-        </is>
-      </c>
-      <c r="C56" s="20" t="inlineStr"/>
-      <c r="D56" s="20" t="inlineStr">
-        <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E56" s="20" t="inlineStr">
-        <is>
-          <t>topic_0769</t>
-        </is>
-      </c>
-      <c r="F56" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_0769</t>
-        </is>
-      </c>
+          <t>Network Isolation</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>Non-egress boundaries, air-gapped artifact staging, localized cloud VPC containers, and firewalled local registries.</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr"/>
+      <c r="E56" s="20" t="inlineStr"/>
+      <c r="F56" s="20" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="20" t="inlineStr">
@@ -4914,10 +4898,14 @@
       </c>
       <c r="B57" s="20" t="inlineStr">
         <is>
-          <t>Model selection</t>
-        </is>
-      </c>
-      <c r="C57" s="20" t="inlineStr"/>
+          <t>Infrastructure Security</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>For on-prem LLM deployments, it captures the security of the compute stack as well as the data pipelines</t>
+        </is>
+      </c>
       <c r="D57" s="20" t="inlineStr"/>
       <c r="E57" s="20" t="inlineStr"/>
       <c r="F57" s="20" t="inlineStr"/>
@@ -4930,25 +4918,17 @@
       </c>
       <c r="B58" s="20" t="inlineStr">
         <is>
-          <t>Evaluation</t>
-        </is>
-      </c>
-      <c r="C58" s="20" t="inlineStr"/>
-      <c r="D58" s="20" t="inlineStr">
-        <is>
-          <t>ACM-CCS</t>
-        </is>
-      </c>
-      <c r="E58" s="20" t="inlineStr">
-        <is>
-          <t>Software and its engineering~Software verification and validation~Software testing and debugging</t>
-        </is>
-      </c>
-      <c r="F58" s="20" t="inlineStr">
-        <is>
-          <t>https://dl.acm.org/ccs</t>
-        </is>
-      </c>
+          <t>Self‑hosted AI</t>
+        </is>
+      </c>
+      <c r="C58" s="20" t="inlineStr">
+        <is>
+          <t>Self‑hosted, open‑weights models in contrast to API‑based models like OpenAI, Anthropic, or Gemini</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="inlineStr"/>
+      <c r="E58" s="20" t="inlineStr"/>
+      <c r="F58" s="20" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="20" t="inlineStr">
@@ -4958,17 +4938,29 @@
       </c>
       <c r="B59" s="20" t="inlineStr">
         <is>
-          <t>Compute Infrastructure</t>
+          <t>Data Protection</t>
         </is>
       </c>
       <c r="C59" s="20" t="inlineStr">
         <is>
-          <t>Physical node topologies, hardware constraints, VRAM bounds, and localized compute execution profiles.</t>
-        </is>
-      </c>
-      <c r="D59" s="20" t="inlineStr"/>
-      <c r="E59" s="20" t="inlineStr"/>
-      <c r="F59" s="20" t="inlineStr"/>
+          <t>Safeguarding sensitive data specifically. Distinct from the broader Security term.</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>topic_4044</t>
+        </is>
+      </c>
+      <c r="F59" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_4044</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="20" t="inlineStr">
@@ -4978,17 +4970,29 @@
       </c>
       <c r="B60" s="20" t="inlineStr">
         <is>
-          <t>Network Isolation</t>
+          <t>FAIR data</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr">
         <is>
-          <t>Non-egress boundaries, air-gapped artifact staging, localized cloud VPC containers, and firewalled local registries.</t>
-        </is>
-      </c>
-      <c r="D60" s="20" t="inlineStr"/>
-      <c r="E60" s="20" t="inlineStr"/>
-      <c r="F60" s="20" t="inlineStr"/>
+          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>topic_4012</t>
+        </is>
+      </c>
+      <c r="F60" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_4012</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="20" t="inlineStr">
@@ -4998,17 +5002,25 @@
       </c>
       <c r="B61" s="20" t="inlineStr">
         <is>
-          <t>Infrastructure Security</t>
-        </is>
-      </c>
-      <c r="C61" s="20" t="inlineStr">
-        <is>
-          <t>For on-prem LLM deployments, it captures the security of the compute stack as well as the data pipelines</t>
-        </is>
-      </c>
-      <c r="D61" s="20" t="inlineStr"/>
-      <c r="E61" s="20" t="inlineStr"/>
-      <c r="F61" s="20" t="inlineStr"/>
+          <t>Data quality management</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr"/>
+      <c r="D61" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>topic_3572</t>
+        </is>
+      </c>
+      <c r="F61" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_3572</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="20" t="inlineStr">
@@ -5018,17 +5030,25 @@
       </c>
       <c r="B62" s="20" t="inlineStr">
         <is>
-          <t>Self‑hosted AI</t>
-        </is>
-      </c>
-      <c r="C62" s="20" t="inlineStr">
-        <is>
-          <t>Self‑hosted, open‑weights models in contrast to API‑based models like OpenAI, Anthropic, or Gemini</t>
-        </is>
-      </c>
-      <c r="D62" s="20" t="inlineStr"/>
-      <c r="E62" s="20" t="inlineStr"/>
-      <c r="F62" s="20" t="inlineStr"/>
+          <t>Data curation and archival</t>
+        </is>
+      </c>
+      <c r="C62" s="20" t="inlineStr"/>
+      <c r="D62" s="20" t="inlineStr">
+        <is>
+          <t>EDAM</t>
+        </is>
+      </c>
+      <c r="E62" s="20" t="inlineStr">
+        <is>
+          <t>topic_0219</t>
+        </is>
+      </c>
+      <c r="F62" s="20" t="inlineStr">
+        <is>
+          <t>http://edamontology.org/topic_0219</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="20" t="inlineStr">
@@ -5038,14 +5058,10 @@
       </c>
       <c r="B63" s="20" t="inlineStr">
         <is>
-          <t>Data Protection</t>
-        </is>
-      </c>
-      <c r="C63" s="20" t="inlineStr">
-        <is>
-          <t>Safeguarding sensitive data specifically. Distinct from the broader Security term.</t>
-        </is>
-      </c>
+          <t>Data integration and warehousing</t>
+        </is>
+      </c>
+      <c r="C63" s="20" t="inlineStr"/>
       <c r="D63" s="20" t="inlineStr">
         <is>
           <t>EDAM</t>
@@ -5053,12 +5069,12 @@
       </c>
       <c r="E63" s="20" t="inlineStr">
         <is>
-          <t>topic_4044</t>
+          <t>topic_3366</t>
         </is>
       </c>
       <c r="F63" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_4044</t>
+          <t>http://edamontology.org/topic_3366</t>
         </is>
       </c>
     </row>
@@ -5070,14 +5086,10 @@
       </c>
       <c r="B64" s="20" t="inlineStr">
         <is>
-          <t>FAIR data</t>
-        </is>
-      </c>
-      <c r="C64" s="20" t="inlineStr">
-        <is>
-          <t>Findable, Accessible, Interoperable, Reusable data principles.</t>
-        </is>
-      </c>
+          <t>Data architecture, analysis and design</t>
+        </is>
+      </c>
+      <c r="C64" s="20" t="inlineStr"/>
       <c r="D64" s="20" t="inlineStr">
         <is>
           <t>EDAM</t>
@@ -5085,12 +5097,12 @@
       </c>
       <c r="E64" s="20" t="inlineStr">
         <is>
-          <t>topic_4012</t>
+          <t>topic_3365</t>
         </is>
       </c>
       <c r="F64" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_4012</t>
+          <t>http://edamontology.org/topic_3365</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5114,7 @@
       </c>
       <c r="B65" s="20" t="inlineStr">
         <is>
-          <t>Data quality management</t>
+          <t>Data identity and mapping</t>
         </is>
       </c>
       <c r="C65" s="20" t="inlineStr"/>
@@ -5113,12 +5125,12 @@
       </c>
       <c r="E65" s="20" t="inlineStr">
         <is>
-          <t>topic_3572</t>
+          <t>topic_3345</t>
         </is>
       </c>
       <c r="F65" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_3572</t>
+          <t>http://edamontology.org/topic_3345</t>
         </is>
       </c>
     </row>
@@ -5130,7 +5142,7 @@
       </c>
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>Data curation and archival</t>
+          <t>Data rescue</t>
         </is>
       </c>
       <c r="C66" s="20" t="inlineStr"/>
@@ -5141,12 +5153,12 @@
       </c>
       <c r="E66" s="20" t="inlineStr">
         <is>
-          <t>topic_0219</t>
+          <t>topic_4011</t>
         </is>
       </c>
       <c r="F66" s="20" t="inlineStr">
         <is>
-          <t>http://edamontology.org/topic_0219</t>
+          <t>http://edamontology.org/topic_4011</t>
         </is>
       </c>
     </row>
@@ -5158,25 +5170,21 @@
       </c>
       <c r="B67" s="20" t="inlineStr">
         <is>
-          <t>Data integration and warehousing</t>
-        </is>
-      </c>
-      <c r="C67" s="20" t="inlineStr"/>
+          <t>Valid and Reliable</t>
+        </is>
+      </c>
+      <c r="C67" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D67" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E67" s="20" t="inlineStr">
-        <is>
-          <t>topic_3366</t>
-        </is>
-      </c>
-      <c r="F67" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3366</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E67" s="20" t="inlineStr"/>
+      <c r="F67" s="20" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="20" t="inlineStr">
@@ -5186,25 +5194,21 @@
       </c>
       <c r="B68" s="20" t="inlineStr">
         <is>
-          <t>Data architecture, analysis and design</t>
-        </is>
-      </c>
-      <c r="C68" s="20" t="inlineStr"/>
+          <t>Safe</t>
+        </is>
+      </c>
+      <c r="C68" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D68" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E68" s="20" t="inlineStr">
-        <is>
-          <t>topic_3365</t>
-        </is>
-      </c>
-      <c r="F68" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3365</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E68" s="20" t="inlineStr"/>
+      <c r="F68" s="20" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="20" t="inlineStr">
@@ -5214,25 +5218,21 @@
       </c>
       <c r="B69" s="20" t="inlineStr">
         <is>
-          <t>Data identity and mapping</t>
-        </is>
-      </c>
-      <c r="C69" s="20" t="inlineStr"/>
+          <t>Secure and Resilient</t>
+        </is>
+      </c>
+      <c r="C69" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D69" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E69" s="20" t="inlineStr">
-        <is>
-          <t>topic_3345</t>
-        </is>
-      </c>
-      <c r="F69" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_3345</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E69" s="20" t="inlineStr"/>
+      <c r="F69" s="20" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="20" t="inlineStr">
@@ -5242,25 +5242,21 @@
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>Data rescue</t>
-        </is>
-      </c>
-      <c r="C70" s="20" t="inlineStr"/>
+          <t>Accountable and Transparent</t>
+        </is>
+      </c>
+      <c r="C70" s="20" t="inlineStr">
+        <is>
+          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+        </is>
+      </c>
       <c r="D70" s="20" t="inlineStr">
         <is>
-          <t>EDAM</t>
-        </is>
-      </c>
-      <c r="E70" s="20" t="inlineStr">
-        <is>
-          <t>topic_4011</t>
-        </is>
-      </c>
-      <c r="F70" s="20" t="inlineStr">
-        <is>
-          <t>http://edamontology.org/topic_4011</t>
-        </is>
-      </c>
+          <t>NIST-AI-RMF</t>
+        </is>
+      </c>
+      <c r="E70" s="20" t="inlineStr"/>
+      <c r="F70" s="20" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="20" t="inlineStr">
@@ -5270,7 +5266,7 @@
       </c>
       <c r="B71" s="20" t="inlineStr">
         <is>
-          <t>Valid and Reliable</t>
+          <t>Explainable and Interpretable</t>
         </is>
       </c>
       <c r="C71" s="20" t="inlineStr">
@@ -5294,7 +5290,7 @@
       </c>
       <c r="B72" s="20" t="inlineStr">
         <is>
-          <t>Safe</t>
+          <t>Privacy-Enhanced</t>
         </is>
       </c>
       <c r="C72" s="20" t="inlineStr">
@@ -5318,12 +5314,12 @@
       </c>
       <c r="B73" s="20" t="inlineStr">
         <is>
-          <t>Secure and Resilient</t>
+          <t>Fair (harmful bias managed)</t>
         </is>
       </c>
       <c r="C73" s="20" t="inlineStr">
         <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
+          <t>NIST AI RMF trustworthy-AI characteristic: algorithmic non-discrimination. NOT the same as 'FAIR data'.</t>
         </is>
       </c>
       <c r="D73" s="20" t="inlineStr">
@@ -5337,162 +5333,66 @@
     <row r="74">
       <c r="A74" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B74" s="20" t="inlineStr">
         <is>
-          <t>Accountable and Transparent</t>
-        </is>
-      </c>
-      <c r="C74" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D74" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr"/>
+      <c r="D74" s="20" t="inlineStr"/>
       <c r="E74" s="20" t="inlineStr"/>
       <c r="F74" s="20" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B75" s="20" t="inlineStr">
         <is>
-          <t>Explainable and Interpretable</t>
-        </is>
-      </c>
-      <c r="C75" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D75" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="C75" s="20" t="inlineStr"/>
+      <c r="D75" s="20" t="inlineStr"/>
       <c r="E75" s="20" t="inlineStr"/>
       <c r="F75" s="20" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B76" s="20" t="inlineStr">
         <is>
-          <t>Privacy-Enhanced</t>
-        </is>
-      </c>
-      <c r="C76" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic.</t>
-        </is>
-      </c>
-      <c r="D76" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr"/>
+      <c r="D76" s="20" t="inlineStr"/>
       <c r="E76" s="20" t="inlineStr"/>
       <c r="F76" s="20" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="20" t="inlineStr">
         <is>
-          <t>Topic Focus</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="B77" s="20" t="inlineStr">
         <is>
-          <t>Fair (harmful bias managed)</t>
-        </is>
-      </c>
-      <c r="C77" s="20" t="inlineStr">
-        <is>
-          <t>NIST AI RMF trustworthy-AI characteristic: algorithmic non-discrimination. NOT the same as 'FAIR data'.</t>
-        </is>
-      </c>
-      <c r="D77" s="20" t="inlineStr">
-        <is>
-          <t>NIST-AI-RMF</t>
-        </is>
-      </c>
+          <t>Deprecated</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="inlineStr"/>
+      <c r="D77" s="20" t="inlineStr"/>
       <c r="E77" s="20" t="inlineStr"/>
       <c r="F77" s="20" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B78" s="20" t="inlineStr">
-        <is>
-          <t>Emerging</t>
-        </is>
-      </c>
-      <c r="C78" s="20" t="inlineStr"/>
-      <c r="D78" s="20" t="inlineStr"/>
-      <c r="E78" s="20" t="inlineStr"/>
-      <c r="F78" s="20" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B79" s="20" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="C79" s="20" t="inlineStr"/>
-      <c r="D79" s="20" t="inlineStr"/>
-      <c r="E79" s="20" t="inlineStr"/>
-      <c r="F79" s="20" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B80" s="20" t="inlineStr">
-        <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="C80" s="20" t="inlineStr"/>
-      <c r="D80" s="20" t="inlineStr"/>
-      <c r="E80" s="20" t="inlineStr"/>
-      <c r="F80" s="20" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="20" t="inlineStr">
-        <is>
-          <t>Maturity Level</t>
-        </is>
-      </c>
-      <c r="B81" s="20" t="inlineStr">
-        <is>
-          <t>Deprecated</t>
-        </is>
-      </c>
-      <c r="C81" s="20" t="inlineStr"/>
-      <c r="D81" s="20" t="inlineStr"/>
-      <c r="E81" s="20" t="inlineStr"/>
-      <c r="F81" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5624,27 +5524,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>Schema.org</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>Schema.org (CreativeWork hierarchy)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>current</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>https://schema.org/CreativeWork</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>Universal web-metadata vocabulary. Exact-type matches applied directly (e.g. APIReference, BlogPosting, ScholarlyArticle, SoftwareSourceCode, Dataset). For highly specific AI-radar terms with no exact schema.org type, the broader parent type is applied instead (e.g. several terms map to TechArticle) -- this is schema.org's own intended usage pattern (broad type + a custom category property), not a forced fit, but it means several distinct Resource Type terms intentionally share one Ontology ID here, unlike EDAM/ACM-CCS/NIST-AI-RMF where each backed term has its own distinct match.</t>
         </is>

</xml_diff>

<commit_message>
Stamp verification: PR #23
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -2482,8 +2482,14 @@
           <t>Lenovo Press</t>
         </is>
       </c>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="1" t="n"/>
+      <c r="E29" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>@pbuendia</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>@biddyman11</t>
@@ -2552,8 +2558,14 @@
           <t xml:space="preserve">Coalition for Secure AI (CoSAI) </t>
         </is>
       </c>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="1" t="n"/>
+      <c r="E30" s="9" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>@pbuendia</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>@biddyman11</t>

</xml_diff>

<commit_message>
Stamp verification: PR #25
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -2482,8 +2482,14 @@
           <t>Lenovo Press</t>
         </is>
       </c>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="1" t="n"/>
+      <c r="E29" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F29" s="1" t="inlineStr">
+        <is>
+          <t>@pbuendia</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>@biddyman11</t>
@@ -2552,8 +2558,14 @@
           <t xml:space="preserve">Coalition for Secure AI (CoSAI) </t>
         </is>
       </c>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="1" t="n"/>
+      <c r="E30" s="9" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F30" s="1" t="inlineStr">
+        <is>
+          <t>@pbuendia</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>@biddyman11</t>

</xml_diff>

<commit_message>
Stamp verification: PR #27
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -1184,6 +1184,14 @@
           <t>GitHub</t>
         </is>
       </c>
+      <c r="E4" s="4" t="n">
+        <v>46262</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>@pbuendia</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>@biddyman11</t>

</xml_diff>

<commit_message>
Add ALAF checklist mapping column; update radar; add Google Drive mirror
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1515" yWindow="1515" windowWidth="24705" windowHeight="12345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Knowledgebase" sheetId="1" state="visible" r:id="rId1"/>
@@ -14,15 +15,14 @@
     <sheet name="Standards" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -33,14 +33,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <color rgb="FF0563C1"/>
-      <sz val="11"/>
       <u val="single"/>
     </font>
   </fonts>
@@ -64,22 +60,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="59">
+  <dxfs count="16">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFDD7E6B"/>
-          <bgColor rgb="FFDD7E6B"/>
+          <fgColor rgb="FFD9D2E9"/>
+          <bgColor rgb="FFD9D2E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -94,6 +97,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFB4A7D6"/>
+          <bgColor rgb="FFB4A7D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFE599"/>
           <bgColor rgb="FFFFE599"/>
         </patternFill>
@@ -102,8 +113,72 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC9DAF8"/>
+          <bgColor rgb="FFC9DAF8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD0E0E3"/>
+          <bgColor rgb="FFD0E0E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE5CD"/>
+          <bgColor rgb="FFFCE5CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCFE2F3"/>
+          <bgColor rgb="FFCFE2F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAD1DC"/>
+          <bgColor rgb="FFEAD1DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB6D7A8"/>
+          <bgColor rgb="FFB6D7A8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -118,432 +193,8 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFB6D7A8"/>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEAD1DC"/>
-          <bgColor rgb="FFEAD1DC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCFE2F3"/>
-          <bgColor rgb="FFCFE2F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE5CD"/>
-          <bgColor rgb="FFFCE5CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD0E0E3"/>
-          <bgColor rgb="FFD0E0E3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC9DAF8"/>
-          <bgColor rgb="FFC9DAF8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEA9999"/>
-          <bgColor rgb="FFEA9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9EAD3"/>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF4CCCC"/>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFE599"/>
-          <bgColor rgb="FFFFE599"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB4A7D6"/>
-          <bgColor rgb="FFB4A7D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA4C2F4"/>
-          <bgColor rgb="FFA4C2F4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D2E9"/>
-          <bgColor rgb="FFD9D2E9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFDD7E6B"/>
           <bgColor rgb="FFDD7E6B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA4C2F4"/>
-          <bgColor rgb="FFA4C2F4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFE599"/>
-          <bgColor rgb="FFFFE599"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE06666"/>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB6D7A8"/>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEAD1DC"/>
-          <bgColor rgb="FFEAD1DC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCFE2F3"/>
-          <bgColor rgb="FFCFE2F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE5CD"/>
-          <bgColor rgb="FFFCE5CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD0E0E3"/>
-          <bgColor rgb="FFD0E0E3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC9DAF8"/>
-          <bgColor rgb="FFC9DAF8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEA9999"/>
-          <bgColor rgb="FFEA9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9EAD3"/>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF4CCCC"/>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFE599"/>
-          <bgColor rgb="FFFFE599"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB4A7D6"/>
-          <bgColor rgb="FFB4A7D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA4C2F4"/>
-          <bgColor rgb="FFA4C2F4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D2E9"/>
-          <bgColor rgb="FFD9D2E9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDD7E6B"/>
-          <bgColor rgb="FFDD7E6B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA4C2F4"/>
-          <bgColor rgb="FFA4C2F4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFE599"/>
-          <bgColor rgb="FFFFE599"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE06666"/>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB6D7A8"/>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEAD1DC"/>
-          <bgColor rgb="FFEAD1DC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCFE2F3"/>
-          <bgColor rgb="FFCFE2F3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFCE5CD"/>
-          <bgColor rgb="FFFCE5CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD0E0E3"/>
-          <bgColor rgb="FFD0E0E3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC9DAF8"/>
-          <bgColor rgb="FFC9DAF8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEA9999"/>
-          <bgColor rgb="FFEA9999"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9EAD3"/>
-          <bgColor rgb="FFD9EAD3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF4CCCC"/>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFE599"/>
-          <bgColor rgb="FFFFE599"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB4A7D6"/>
-          <bgColor rgb="FFB4A7D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFA4C2F4"/>
-          <bgColor rgb="FFA4C2F4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D2E9"/>
-          <bgColor rgb="FFD9D2E9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -909,12 +560,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="26.5703125" customWidth="1" min="2" max="2"/>
-    <col width="37.28515625" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -925,10 +576,11 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="26" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="43" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="43" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="23" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -999,20 +651,25 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>ALAF Checklist Mapping</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Relevance to Research Cyberinfrastructure</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Maturity Level</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Discovery Date</t>
         </is>
@@ -1073,22 +730,22 @@
           <t>Architecture;Implementation;Deployment</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>IDE integration for agentic workflows</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Canonical reference for VS Code agent capabilities.</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="R2" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -1149,17 +806,17 @@
           <t>Workflows;Implementation</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Makes data outputs FAIR at the point of publication</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="n">
+      <c r="R3" s="3" t="n">
         <v>46168</v>
       </c>
     </row>
@@ -1184,7 +841,7 @@
           <t>GitHub</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="3" t="n">
         <v>46262</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -1197,7 +854,7 @@
           <t>@biddyman11</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="3" t="n">
         <v>46262</v>
       </c>
       <c r="K4" t="inlineStr">
@@ -1215,22 +872,22 @@
           <t>Architecture;Governance;Security</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Relevant for CI/CD and code-review automation</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Strong alignment with developer workflows.</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="n">
+      <c r="R4" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -1275,22 +932,22 @@
           <t>Architecture;Implementation</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Key for interoperable agent tools</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Fast-moving ecosystem.</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="n">
+      <c r="R5" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -1335,22 +992,22 @@
           <t>Architecture;Governance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Critical for cross-platform agent interoperability</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Becoming a de facto standard.</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="n">
+      <c r="R6" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -1409,22 +1066,22 @@
           <t>Architecture;Governance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Integration between LLM applications and external data sources and tools</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Strong safety emphasis.</t>
         </is>
       </c>
-      <c r="Q7" s="3" t="n">
+      <c r="R7" s="3" t="n">
         <v>45962</v>
       </c>
     </row>
@@ -1485,50 +1142,53 @@
           <t>Implementation;Security;Deployment</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Helps teams move prototypes to production</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Technical guide to the operational life cycle of AI agents, focusing on deployment &amp; security</t>
         </is>
       </c>
-      <c r="Q8" s="3" t="n">
+      <c r="R8" s="3" t="n">
         <v>45975</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>bfda8877</t>
+          <t>f488464f</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Google Vertex AI Agents Overview</t>
+          <t>HuggingFace Agents Documentation</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/vertex-ai/docs/agents</t>
+          <t>https://huggingface.co/docs/hub/en/agents</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Paty Buendia</t>
-        </is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>46265</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1537,52 +1197,52 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Agent frameworks;Orchestration</t>
+          <t>Tools;Skills;Model Integration</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Architecture;Deployment</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Useful for cloud-based scientific workflows</t>
+          <t>Architecture;Implementation</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Useful for open-source agent experimentation</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Strong enterprise alignment.</t>
-        </is>
-      </c>
-      <c r="Q9" s="3" t="n">
-        <v>46113</v>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Rapidly evolving.</t>
+        </is>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>46082</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>f488464f</t>
+          <t>dbe3741e</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HuggingFace Agents Documentation</t>
+          <t>LangChain Agents Overview</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/docs/agents</t>
+          <t>https://python.langchain.com/docs/modules/agents</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>LangChain</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1597,7 +1257,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Tools;Skills;Model Integration</t>
+          <t>Tools;Skills;Multi-Agent Patterns</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1605,44 +1265,44 @@
           <t>Architecture;Implementation</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Useful for open-source agent experimentation</t>
-        </is>
-      </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Relevant for workflow prototyping</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Rapidly evolving.</t>
-        </is>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>46082</v>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Widely used in research.</t>
+        </is>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dbe3741e</t>
+          <t>ddd42289</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LangChain Agents Overview</t>
+          <t>LlamaIndex Agents</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>https://python.langchain.com/docs/modules/agents</t>
+          <t>https://docs.llamaindex.ai/en/stable/agent/</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LangChain</t>
+          <t>LlamaIndex</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1657,52 +1317,60 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Tools;Skills;Multi-Agent Patterns</t>
+          <t>Tools;Skills;Retrieval Agents</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Architecture;Implementation</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Relevant for workflow prototyping</t>
+          <t>Architecture;Governance</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
+          <t>Useful for data-rich research platforms</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Widely used in research.</t>
-        </is>
-      </c>
-      <c r="Q11" s="3" t="n">
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Strong retrieval-centric design.</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ddd42289</t>
+          <t>c7e95f61</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LlamaIndex Agents</t>
+          <t>Dagster Automation/Agent Patterns</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://docs.llamaindex.ai/en/stable/agent/</t>
+          <t>https://docs.dagster.io/getting-started/ai-tools</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LlamaIndex</t>
+          <t>Dagster Labs</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>46082</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Paty Buendia</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1710,6 +1378,14 @@
           <t>Paty Buendia</t>
         </is>
       </c>
+      <c r="H12" s="3" t="n">
+        <v>46082</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1.3.15</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Documentation</t>
@@ -1717,73 +1393,57 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Tools;Skills;Retrieval Agents</t>
+          <t>Workflow Automation;Orchestration</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Architecture;Governance</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Useful for data-rich research platforms</t>
+          <t>Architecture;Deployment</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Relevant for scientific pipelines</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Strong retrieval-centric design.</t>
-        </is>
-      </c>
-      <c r="Q12" s="3" t="n">
-        <v>46113</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Strong reproducibility focus.</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>46082</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>c7e95f61</t>
+          <t>73426de0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dagster Automation/Agent Patterns</t>
+          <t>Prefect Automations/Agents</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>https://docs.dagster.io/getting-started/ai-tools</t>
+          <t>https://docs.prefect.io/latest/concepts/automations/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Dagster Labs</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>46082</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Paty Buendia</t>
+          <t>Prefect</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Paty Buendia</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="n">
-        <v>46082</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>1.3.15</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1793,57 +1453,57 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Workflow Automation;Orchestration</t>
+          <t>Workflow Agents;Triggers</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Architecture;Deployment</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Relevant for scientific pipelines</t>
+          <t>Implementation;Deployment</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
+          <t>Useful for data processing pipelines</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Strong reproducibility focus.</t>
-        </is>
-      </c>
-      <c r="Q13" s="3" t="n">
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Good hybrid cloud/HPC support.</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="n">
         <v>46082</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>73426de0</t>
+          <t>3294a13f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prefect Automations/Agents</t>
+          <t>Jupyter AI</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://docs.prefect.io/latest/concepts/automations/</t>
+          <t>https://jupyter-ai.readthedocs.io</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Prefect</t>
+          <t>Project Jupyter</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1853,177 +1513,177 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Workflow Agents;Triggers</t>
+          <t>Notebook Agents;Workflow Automation</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Implementation;Deployment</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>Useful for data processing pipelines</t>
+          <t>Implementation;Data governance</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Mature</t>
+          <t>Relevant for research notebooks</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Good hybrid cloud/HPC support.</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="n">
-        <v>46082</v>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Strong alignment with scientific workflows.</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3294a13f</t>
+          <t>f51ea180</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jupyter AI</t>
+          <t>Anthropic Tools API</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>https://jupyter-ai.readthedocs.io</t>
+          <t>https://docs.anthropic.com/en/docs/tools</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Project Jupyter</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>API Reference</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Notebook Agents;Workflow Automation</t>
+          <t>Tools;Skills</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Implementation;Data governance</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Relevant for research notebooks</t>
+          <t>Architecture;Security</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
+          <t>Useful for safe tool-calling agents</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Strong alignment with scientific workflows.</t>
-        </is>
-      </c>
-      <c r="Q15" s="3" t="n">
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Strong safety posture.</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>f51ea180</t>
+          <t>89f36cc1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Anthropic Tools API</t>
+          <t>Microsoft Semantic Kernel Agents</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://docs.anthropic.com/en/docs/tools</t>
+          <t>https://learn.microsoft.com/semantic-kernel/agents</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>API Reference</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Tools;Skills</t>
+          <t>Skills;Tools;Orchestration</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Architecture;Security</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Useful for safe tool-calling agents</t>
+          <t>Architecture;Implementation</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Useful for enterprise-grade agent workflows</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Strong safety posture.</t>
-        </is>
-      </c>
-      <c r="Q16" s="3" t="n">
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Strong .NET + Python support.</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>89f36cc1</t>
+          <t>4ccfda21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Microsoft Semantic Kernel Agents</t>
+          <t>HuggingFace Inference Endpoints</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>https://learn.microsoft.com/semantic-kernel/agents</t>
+          <t>https://huggingface.co/inference-endpoints</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>HuggingFace</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2033,57 +1693,57 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Skills;Tools;Orchestration</t>
+          <t>Model Integration;Tool-Ready Endpoints</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Architecture;Implementation</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Useful for enterprise-grade agent workflows</t>
+          <t>Architecture;Deployment</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Useful for hosted inference in research</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Strong .NET + Python support.</t>
-        </is>
-      </c>
-      <c r="Q17" s="3" t="n">
-        <v>46113</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Good for reproducibility.</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="n">
+        <v>46082</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4ccfda21</t>
+          <t>2e24be4d</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HuggingFace Inference Endpoints</t>
+          <t>OpenAI Evaluations (Evals)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>https://huggingface.co/inference-endpoints</t>
+          <t>https://platform.openai.com/docs/guides/evals</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>HuggingFace</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2093,57 +1753,57 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Model Integration;Tool-Ready Endpoints</t>
+          <t>Evaluation / testing;Safety / guardrails</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Architecture;Deployment</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Useful for hosted inference in research</t>
+          <t>Security;Governance</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Mature</t>
+          <t>Relevant for agent safety in research platforms</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Good for reproducibility.</t>
-        </is>
-      </c>
-      <c r="Q18" s="3" t="n">
-        <v>46082</v>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Useful for risk assessment.</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2e24be4d</t>
+          <t>6b9e7398</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>OpenAI Evaluations (Evals)</t>
+          <t>Anthropic Safety Guidelines</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>https://platform.openai.com/docs/guides/evals</t>
+          <t>https://docs.anthropic.com/en/docs/safety</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2153,242 +1813,257 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Evaluation / testing;Safety / guardrails</t>
+          <t>Safety / guardrails;Safe Tool Use</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Security;Governance</t>
+          <t>Governance;Security</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Relevant for agent safety in research platforms</t>
+          <t>Agent Manifesto</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Useful for research governance teams</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Useful for risk assessment.</t>
-        </is>
-      </c>
-      <c r="Q19" s="3" t="n">
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Strong alignment with institutional risk controls.</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6b9e7398</t>
+          <t>69804f39</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Anthropic Safety Guidelines</t>
+          <t>Microsoft Responsible AI Standard</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>https://docs.anthropic.com/en/docs/safety</t>
+          <t>https://www.microsoft.com/ai/responsible-ai</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Governance Guidance</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Safety / guardrails;Safe Tool Use</t>
+          <t>Safety / guardrails;Governance;Risk Controls</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Governance;Security</t>
+          <t>Data governance;Security</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Useful for research governance teams</t>
+          <t>Agent Manifesto;Human Approval Gate</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
+          <t>Relevant for institutional AI governance</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>Strong alignment with institutional risk controls.</t>
-        </is>
-      </c>
-      <c r="Q20" s="3" t="n">
-        <v>46113</v>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Widely adopted governance framework.</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="n">
+        <v>45992</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>69804f39</t>
+          <t>3758624e</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Microsoft Responsible AI Standard</t>
+          <t>vLLM Documentation</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>https://www.microsoft.com/ai/responsible-ai</t>
+          <t>https://docs.vllm.ai</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>vLLM Project Team</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Governance Guidance</t>
+          <t>Inference Framework</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Safety / guardrails;Governance;Risk Controls</t>
+          <t>Deployment patterns;Tools</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Data governance;Security</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Relevant for institutional AI governance</t>
+          <t>Self‑hosted AI;Architecture;Implementation;Deployment</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
+          <t>High (Industry-standard VPC runtime engine)</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>Widely adopted governance framework.</t>
-        </is>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>45992</v>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Essential for secure TLAs via PagedAttention and FP8/AWQ optimization. Capabilities: Parallel sampling &amp; tool-calling.</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3758624e</t>
+          <t>8a50b5eb</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>vLLM Documentation</t>
+          <t>Ollama Documentation</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>https://docs.vllm.ai</t>
+          <t>https://github.com/ollama/ollama</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>vLLM Project Team</t>
+          <t>Ollama Community</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Inference Framework</t>
+          <t>Local Application Sandbox</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Deployment patterns;Tools</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Architecture;Implementation;Deployment</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>High (Industry-standard VPC runtime engine)</t>
+          <t>Self‑hosted AI;Implementation;Deployment</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
+          <t>Medium-High (Local workstation co-pilot)</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>Essential for secure TLAs via PagedAttention and FP8/AWQ optimization. Capabilities: Parallel sampling &amp; tool-calling.</t>
-        </is>
-      </c>
-      <c r="Q22" s="3" t="n">
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Eliminates network dependency errors by cleanly bundling open model weights. Capabilities: Local embedding &amp; zero-config tools.</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="n">
         <v>46113</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>8a50b5eb</t>
+          <t>763797cd</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ollama Documentation</t>
+          <t xml:space="preserve">Llama.cpp </t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/ollama/ollama</t>
+          <t>https://github.com/ggerganov/llama.cpp</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ollama Community</t>
+          <t>Georgi Gerganov</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>b9253</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Local Application Sandbox</t>
+          <t>Github Code Repository</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2398,182 +2073,182 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Implementation;Deployment</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Medium-High (Local workstation co-pilot)</t>
+          <t>Self‑hosted AI;Architecture;Implementation;Deployment</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
+          <t>High (Enables reasoning on variable local hardware)</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>Eliminates network dependency errors by cleanly bundling open model weights. Capabilities: Local embedding &amp; zero-config tools.</t>
-        </is>
-      </c>
-      <c r="Q23" s="3" t="n">
-        <v>46113</v>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Grammar constraints ensure localized agentic pipelines always return valid JSON/code. Capabilities: Grammar-based constrained sampling.</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="n">
+        <v>46162</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>763797cd</t>
+          <t>2d2470f7</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Llama.cpp </t>
+          <t>Open WebUI Documentation</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/ggerganov/llama.cpp</t>
+          <t>https://docs.openwebui.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Georgi Gerganov</t>
+          <t>Open WebUI Core Team</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>claude</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>b9253</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Github Code Repository</t>
+          <t>Enterprise Control Interface</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Deployment patterns</t>
+          <t>Retrieval</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Architecture;Implementation;Deployment</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>High (Enables reasoning on variable local hardware)</t>
+          <t>Self‑hosted AI;Implementation;Deployment</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
+          <t>High (Enterprise-grade firewall interface)</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>Grammar constraints ensure localized agentic pipelines always return valid JSON/code. Capabilities: Grammar-based constrained sampling.</t>
-        </is>
-      </c>
-      <c r="Q24" s="3" t="n">
-        <v>46162</v>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Solves local file parsing/RAG bottlenecks entirely within secure client networks. Capabilities: Local RAG pipelines &amp; offline functions.</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="n">
+        <v>46113</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2d2470f7</t>
+          <t>eb79015c</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Open WebUI Documentation</t>
+          <t>NVIDIA NIM Air-Gap Deployment Guide</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>https://docs.openwebui.com</t>
+          <t>https://docs.nvidia.com/nim/large-language-models/latest/deploy-air-gap.html</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Open WebUI Core Team</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Enterprise Control Interface</t>
+          <t>Reference Architecture</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Retrieval</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Implementation;Deployment</t>
+          <t>Self‑hosted AI;Compute Infrastructure;Implementation;Network Isolation;Infrastructure Security</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>High (Enterprise-grade firewall interface)</t>
+          <t>Remediate Oversharing</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
+          <t>Critical (Standardizes secure distribution of optimized weights)</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>Solves local file parsing/RAG bottlenecks entirely within secure client networks. Capabilities: Local RAG pipelines &amp; offline functions.</t>
-        </is>
-      </c>
-      <c r="Q25" s="3" t="n">
-        <v>46113</v>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Outlines the exact connected-to-disconnected asset transfer workflow for enterprise GPUs. Capabilities: Tensor-parallel caching &amp; optimized tool-calling.</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="n">
+        <v>46150</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>eb79015c</t>
+          <t>80527de7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NVIDIA NIM Air-Gap Deployment Guide</t>
+          <t>Harbor User Documentation</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>https://docs.nvidia.com/nim/large-language-models/latest/deploy-air-gap.html</t>
+          <t>https://goharbor.io/docs/</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Cloud Native Computing Foundation (CNCF)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Reference Architecture</t>
+          <t>Container Registry</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2583,167 +2258,193 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Compute Infrastructure;Implementation;Network Isolation;Infrastructure Security</t>
+          <t>Self‑hosted AI;Implementation;Network Isolation;Infrastructure Security;Governance</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Critical (Standardizes secure distribution of optimized weights)</t>
+          <t>Provenance and Reversibility</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
+          <t>High (Necessary foundation for secure cluster registries)</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>Outlines the exact connected-to-disconnected asset transfer workflow for enterprise GPUs. Capabilities: Tensor-parallel caching &amp; optimized tool-calling.</t>
-        </is>
-      </c>
-      <c r="Q26" s="3" t="n">
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Built-in vulnerability scanning ensures agent images remain clean behind the firewall. Capabilities: Artifact version-locking &amp; immutable tags.</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="n">
         <v>46150</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>80527de7</t>
+          <t>b4b5a468</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Harbor User Documentation</t>
+          <t>AI Engineering Blueprint for On-Premises RAG Systems</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>https://goharbor.io/docs/</t>
+          <t>https://arxiv.org/abs/2604.01395</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Cloud Native Computing Foundation (CNCF)</t>
+          <t>arXiv (2604.01395)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Container Registry</t>
+          <t>Scientific Literature</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Deployment patterns</t>
+          <t>Deployment patterns;Retrieval</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Implementation;Network Isolation;Infrastructure Security;Governance</t>
+          <t>Self‑hosted AI;Infrastructure Security</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>High (Necessary foundation for secure cluster registries)</t>
+          <t>Remediate Oversharing</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Mature</t>
+          <t>High (Academic/industry validated system design blueprint)</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Built-in vulnerability scanning ensures agent images remain clean behind the firewall. Capabilities: Artifact version-locking &amp; immutable tags.</t>
-        </is>
-      </c>
-      <c r="Q27" s="3" t="n">
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Moves past simple how-to guides into formal data isolation and local compliance frameworks. Capabilities: End-to-end local reference applications.</t>
+        </is>
+      </c>
+      <c r="R27" s="3" t="n">
         <v>46150</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>b4b5a468</t>
+          <t>0d0a50a7</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>AI Engineering Blueprint for On-Premises RAG Systems</t>
+          <t>On-Premise vs Cloud: GenAI TCO (2026 Edition)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2604.01395</t>
+          <t xml:space="preserve">https://lenovopress.lenovo.com/lp2368-on-premise-vs-cloud-generative-ai-total-cost-of-ownership-2026-edition </t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>arXiv (2604.01395)</t>
+          <t>Lenovo Press</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>@pbuendia</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>claude</t>
+          <t>@biddyman11</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Scientific Literature</t>
+          <t>Whitepaper</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Deployment patterns;Retrieval</t>
+          <t>Deployment patterns</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Infrastructure Security</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>High (Academic/industry validated system design blueprint)</t>
+          <t>Self‑hosted AI;Architecture;Governance</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>High (Mandatory for spec'ing out server node VRAM limits)</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Moves past simple how-to guides into formal data isolation and local compliance frameworks. Capabilities: End-to-end local reference applications.</t>
-        </is>
-      </c>
-      <c r="Q28" s="3" t="n">
-        <v>46150</v>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Discusses a "Token Economics" framework. Breaks down the "Memory Wall" economics showing an on-prem breakeven velocity of ~4 months. Capabilities: Hardware performance scaling &amp; VRAM sizing.</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>46054</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0d0a50a7</t>
+          <t>359b5ac8</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>On-Premise vs Cloud: GenAI TCO (2026 Edition)</t>
+          <t xml:space="preserve">Coalition for Secure AI (CoSAI) </t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lenovopress.lenovo.com/lp2368-on-premise-vs-cloud-generative-ai-total-cost-of-ownership-2026-edition </t>
+          <t>https://www.coalitionforsecureai.org/</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Lenovo Press</t>
+          <t xml:space="preserve">Coalition for Secure AI (CoSAI) </t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
@@ -2762,81 +2463,84 @@
       <c r="H29" s="3" t="n">
         <v>46259</v>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Whitepaper</t>
+          <t>Security Guidance &amp; Resources</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Deployment patterns</t>
+          <t>Safety / guardrails;Safe Tool Use</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Self‑hosted AI;Architecture;Governance</t>
+          <t>Infrastructure Security;Security</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>High (Mandatory for spec'ing out server node VRAM limits)</t>
+          <t>Agent Manifesto</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Mature</t>
+          <t>Relevant security expertise and best practices for secure AI development and deployment</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Discusses a "Token Economics" framework. Breaks down the "Memory Wall" economics showing an on-prem breakeven velocity of ~4 months. Capabilities: Hardware performance scaling &amp; VRAM sizing.</t>
-        </is>
-      </c>
-      <c r="Q29" s="3" t="n">
-        <v>46054</v>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>The Coalition for Secure AI (CoSAI) is an open ecosystem of AI and security experts. See https://github.com/cosai-oasis/ws2-defenders</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="n">
+        <v>46174</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>359b5ac8</t>
+          <t>5f3954c2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coalition for Secure AI (CoSAI) </t>
+          <t>Anthropic Project Glasswing</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>https://www.coalitionforsecureai.org/</t>
+          <t>https://www.anthropic.com/glasswing</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coalition for Secure AI (CoSAI) </t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>46259</v>
+        <v>46182</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>@pbuendia</t>
+          <t>Paty Buendia</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>@biddyman11</t>
+          <t>Paty Buendia</t>
         </is>
       </c>
       <c r="H30" s="3" t="n">
-        <v>46259</v>
+        <v>46182</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>46119</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -2845,7 +2549,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Safety / guardrails;Safe Tool Use</t>
+          <t>Cybersecurity</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2853,48 +2557,48 @@
           <t>Infrastructure Security;Security</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>Relevant security expertise and best practices for secure AI development and deployment</t>
-        </is>
-      </c>
       <c r="O30" t="inlineStr">
         <is>
+          <t>AI models that find high-severity vulnerabilities</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
           <t>Emerging</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>The Coalition for Secure AI (CoSAI) is an open ecosystem of AI and security experts. See https://github.com/cosai-oasis/ws2-defenders</t>
-        </is>
-      </c>
-      <c r="Q30" s="3" t="n">
-        <v>46174</v>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>See Claude Mythos Preview</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="n">
+        <v>46119</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5f3954c2</t>
+          <t>1c277820</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Anthropic Project Glasswing</t>
+          <t>Docker AI Governance &amp; Sandboxes</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>https://www.anthropic.com/glasswing</t>
+          <t>https://docs.docker.com/ai/sandboxes/governance/org/</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Docker</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>46182</v>
+        <v>46219</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -2907,68 +2611,75 @@
         </is>
       </c>
       <c r="H31" s="3" t="n">
-        <v>46182</v>
-      </c>
-      <c r="J31" s="3" t="n">
-        <v>46119</v>
+        <v>46219</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>0.35.0</t>
+        </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Security Guidance &amp; Resources</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Cybersecurity</t>
+          <t>Sandbox;MCP</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Infrastructure Security;Security</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>AI models that find high-severity vulnerabilities</t>
+          <t>Remediate Oversharing;Human Approval Gate</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Emerging</t>
+          <t>Good AI governance topics</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>See Claude Mythos Preview</t>
-        </is>
-      </c>
-      <c r="Q31" s="3" t="n">
-        <v>46119</v>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>See blog article: https://www.docker.com/blog/the-3cs-a-framework-for-ai-agent-security/</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="n">
+        <v>46213</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1c277820</t>
+          <t>b39dc1d1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Docker AI Governance &amp; Sandboxes</t>
+          <t>Responses API</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>https://docs.docker.com/ai/sandboxes/governance/org/</t>
+          <t>https://developers.openai.com/api/docs/guides/migrate-to-responses</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Docker</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -2981,11 +2692,11 @@
         </is>
       </c>
       <c r="H32" s="3" t="n">
-        <v>46219</v>
+        <v>46220</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>0.35.0</t>
+          <t>GPT-5.6</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2995,56 +2706,56 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Sandbox;MCP</t>
+          <t>Tools;Skills;Retrieval</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Good AI governance topics</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Useful for domain-specific agents</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>See blog article: https://www.docker.com/blog/the-3cs-a-framework-for-ai-agent-security/</t>
-        </is>
-      </c>
-      <c r="Q32" s="3" t="n">
-        <v>46213</v>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>MIgrated from API Assistants  - now deprecated.</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="n">
+        <v>46212</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>b39dc1d1</t>
+          <t>9717f0f1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Responses API</t>
+          <t>OWASP Top 10 for Agentic Applications 2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>https://developers.openai.com/api/docs/guides/migrate-to-responses</t>
+          <t>https://genai.owasp.org/resource/owasp-top-10-for-agentic-applications-for-2026/</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>OWASP GenAI Security Project</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>46220</v>
+        <v>46265</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -3053,117 +2764,198 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Security Guidance &amp; Resources</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Safety / guardrails;Risk Controls;Safe Tool Use;Cybersecurity</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Security;Governance;Secure and Resilient</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Runtime PII Screening;Human Approval Gate</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Threat catalog for autonomous agents; names the risks a research platform must design against</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Ten risk categories (ASI01-ASI10) for agents that plan, hold memory, and call tools, with threats and mitigations for each. Released December 2025, globally peer-reviewed. CC BY-SA 4.0, so it can be adapted with attribution. Initiative: https://github.com/genai-security-project/</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="n">
+        <v>46265</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>c580e5f8</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>NIST AI RMF Playbook</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>https://airc.nist.gov/airmf-resources/playbook/</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>NIST</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>Paty Buendia</t>
         </is>
       </c>
-      <c r="H33" s="3" t="n">
-        <v>46220</v>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>GPT-5.6</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Tools;Skills;Retrieval</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Useful for domain-specific agents</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>Emerging</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>MIgrated from API Assistants  - now deprecated.</t>
-        </is>
-      </c>
-      <c r="Q33" s="3" t="n">
-        <v>46212</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Governance Guidance</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Governance;Risk Controls;Evaluation / testing</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Governance;Accountable and Transparent;Valid and Reliable</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Agent Manifesto;Human Approval Gate;Provenance and Reversibility</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Focuses on 4 functions: Govern, Map, Measure, Manage. The Playbook is the companion document. NIST AI RMF 1.0 is used in this project's own vocabulary </t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Companion to NIST AI RMF 1.0. Voluntary, free, and organised around Govern, Map, Measure and Manage, with suggested actions and references per outcome. Organisations take as many or as few suggestions as apply.</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="n">
+        <v>46265</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E33">
-    <cfRule type="expression" priority="1" dxfId="18">
+  <conditionalFormatting sqref="E2:E34">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>E2&gt;=DATE(2026,5,9)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K33">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+  <conditionalFormatting sqref="K2:K34">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"Documentation"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"API Reference"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="15">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Specification"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"Whitepaper"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="13">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
       <formula>"Scientific Literature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
       <formula>"Governance Guidance"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
       <formula>"Security Guidance &amp; Resources"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
       <formula>"Reference Architecture"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"Container Registry"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
       <formula>"Enterprise Control Interface"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
       <formula>"Inference Framework"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
       <formula>"Local Application Sandbox"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
       <formula>"Github Code Repository"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
       <formula>"Benchmark Collection"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M33">
-    <cfRule type="expression" priority="16" dxfId="3">
+  <conditionalFormatting sqref="M2:M34">
+    <cfRule type="expression" priority="16" dxfId="1">
       <formula>LEN(TRIM(M2))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O33">
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="3">
+  <conditionalFormatting sqref="P2:P34">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="1">
       <formula>"Emerging"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="4">
       <formula>"Research"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="2">
       <formula>"Mature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="15">
       <formula>"Deprecated"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3200,6 +2992,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3211,7 +3004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3228,10 +3021,11 @@
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="43" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="23" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="43" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3307,20 +3101,25 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>ALAF Checklist Mapping</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Relevance to Research Cyberinfrastructure</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Maturity Level</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Discovery Date</t>
         </is>
@@ -3347,127 +3146,195 @@
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="3" t="n"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Paty Buendia</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>API Reference</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Tools;Skills;Retrieval</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Architecture;Implementation</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Useful for domain-specific agents</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Deprecated</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Stable API surface. Migrated to the `Responses API`.</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="n">
         <v>46150</v>
       </c>
-      <c r="F2" t="inlineStr">
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>bfda8877</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Google Vertex AI Agents Overview</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/vertex-ai/docs/agents</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Paty Buendia</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Paty Buendia</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>46150</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>API Reference</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Tools;Skills;Retrieval</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Architecture;Implementation</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Useful for domain-specific agents</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Agent frameworks;Orchestration</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Architecture;Deployment</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Useful for cloud-based scientific workflows</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Deprecated</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Stable API surface.</t>
-        </is>
-      </c>
-      <c r="R2" s="3" t="n">
-        <v>46150</v>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Documentation URL no longer resolves: cloud.google.com/vertex-ai/docs/agents 301-redirects to docs.cloud.google.com/vertex-ai/docs/agents, which returns 404. Google's agent tooling has moved to Agent Builder. Needs a replacement resource.</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>46113</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2">
-    <cfRule type="expression" priority="1" dxfId="18">
+  <conditionalFormatting sqref="E2:E3">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>E2&gt;=DATE(2026,5,9)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L2">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+  <conditionalFormatting sqref="L2:L3">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"Documentation"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"API Reference"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="15">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Specification"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"Whitepaper"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="13">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
       <formula>"Scientific Literature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
       <formula>"Governance Guidance"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
       <formula>"Security Guidance &amp; Resources"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
       <formula>"Reference Architecture"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"Container Registry"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
       <formula>"Enterprise Control Interface"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
       <formula>"Inference Framework"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
       <formula>"Local Application Sandbox"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
       <formula>"Github Code Repository"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
       <formula>"Benchmark Collection"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2">
-    <cfRule type="expression" priority="16" dxfId="3">
+  <conditionalFormatting sqref="N2:N3">
+    <cfRule type="expression" priority="16" dxfId="1">
       <formula>LEN(TRIM(N2))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2">
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="3">
+  <conditionalFormatting sqref="Q2:Q3">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="1">
       <formula>"Emerging"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="4">
       <formula>"Research"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="2">
       <formula>"Mature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="15">
       <formula>"Deprecated"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3479,7 +3346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3494,9 +3361,10 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="23" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3562,15 +3430,20 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>ALAF Checklist Mapping</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Maturity Level</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notes / Key Takeaways</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Discovery Date</t>
         </is>
@@ -3628,17 +3501,17 @@
           <t>Coding Agents</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Evaluates State-Of-The-Art agent performance on multi-million line codebases to assess real-world software engineering capabilities.</t>
         </is>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="P2" s="3" t="n">
         <v>46216</v>
       </c>
     </row>
@@ -3689,17 +3562,17 @@
           <t>Coding Agents</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Papers with Code with State-Of-The-Art (SOTA) Codng Agent Benchmarks</t>
         </is>
       </c>
-      <c r="O3" s="3" t="n">
+      <c r="P3" s="3" t="n">
         <v>46216</v>
       </c>
     </row>
@@ -3744,17 +3617,17 @@
           <t>Coding Agents</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Addresses limitations of original SWE-bench by focusing on long-horizon, complex, multi-file software engineering tasks.</t>
         </is>
       </c>
-      <c r="O4" s="3" t="n">
+      <c r="P4" s="3" t="n">
         <v>46216</v>
       </c>
     </row>
@@ -3794,17 +3667,17 @@
           <t>Coding Agents</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Scalable framework that generates repository-level tasks from live GitHub PRs across 11 programming languages.</t>
         </is>
       </c>
-      <c r="O5" s="3" t="n">
+      <c r="P5" s="3" t="n">
         <v>46216</v>
       </c>
     </row>
@@ -3849,17 +3722,17 @@
           <t>Coding Agents</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Benchmarks agents on hard, realistic tasks within terminal/CLI environments.</t>
         </is>
       </c>
-      <c r="O6" s="3" t="n">
+      <c r="P6" s="3" t="n">
         <v>46216</v>
       </c>
     </row>
@@ -3904,17 +3777,17 @@
           <t>Coding Agents</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Benchmark specifically for evaluating the code review capabilities of AI agents.</t>
         </is>
       </c>
-      <c r="O7" s="3" t="n">
+      <c r="P7" s="3" t="n">
         <v>46216</v>
       </c>
     </row>
@@ -3959,81 +3832,81 @@
           <t>Coding Agents</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Isolates the evaluation of repository exploration, context retrieval, and code localization capabilities.</t>
         </is>
       </c>
-      <c r="O8" s="3" t="n">
+      <c r="P8" s="3" t="n">
         <v>46216</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E8">
-    <cfRule type="expression" priority="1" dxfId="18">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>E2&gt;=DATE(2026,5,9)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K8">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
       <formula>"Documentation"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"API Reference"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="15">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"Specification"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"Whitepaper"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="13">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
       <formula>"Scientific Literature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
       <formula>"Governance Guidance"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
       <formula>"Security Guidance &amp; Resources"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
       <formula>"Reference Architecture"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"Container Registry"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
       <formula>"Enterprise Control Interface"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
       <formula>"Inference Framework"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
       <formula>"Local Application Sandbox"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
       <formula>"Github Code Repository"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
       <formula>"Benchmark Collection"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M8">
-    <cfRule type="cellIs" priority="16" operator="equal" dxfId="3">
+  <conditionalFormatting sqref="N2:N8">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="1">
       <formula>"Emerging"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="4">
       <formula>"Research"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
       <formula>"Mature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="15">
       <formula>"Deprecated"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4056,12 +3929,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="4"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -4480,22 +4354,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Relevance to Research Cyberinfrastructure</t>
+          <t>ALAF Checklist Mapping</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Knowledgebase; Deprecated</t>
+          <t>Knowledgebase; Deprecated; SOTA Coding Agents Benchmarks</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>free_text</t>
+          <t>controlled_multi</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>;</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Free-text note on why this matters to research platforms. Example themes: workflow orchestration, data portal integration, metadata / provenance, multi-agent coordination, HPC / cloud hybrid workflows, reproducibility, federated analysis, user-facing agent interfaces.</t>
+          <t>Which readiness items from the ALAF Checklist this resource helps an organization satisfy. One or more terms, separated by ';'. Blank means the resource is not specific to any checklist item.</t>
         </is>
       </c>
     </row>
@@ -4505,22 +4384,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Maturity Level</t>
+          <t>Relevance to Research Cyberinfrastructure</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Knowledgebase; Deprecated; SOTA Coding Agents Benchmarks</t>
+          <t>Knowledgebase; Deprecated</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>controlled_single</t>
+          <t>free_text</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Not about the website - about the technology described. Helps teams know whether something is stable enough to consider.</t>
+          <t>Free-text note on why this matters to research platforms. Example themes: workflow orchestration, data portal integration, metadata / provenance, multi-agent coordination, HPC / cloud hybrid workflows, reproducibility, federated analysis, user-facing agent interfaces.</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4409,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Notes / Key Takeaways</t>
+          <t>Maturity Level</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4540,12 +4419,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>free_text</t>
+          <t>controlled_single</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Short free-text field: breaking changes, important patterns, new capabilities, relevance to agentic workflows, implications for research platforms. This is where institutional knowledge accumulates.</t>
+          <t>Not about the website - about the technology described. Helps teams know whether something is stable enough to consider.</t>
         </is>
       </c>
     </row>
@@ -4555,20 +4434,45 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>Notes / Key Takeaways</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Knowledgebase; Deprecated; SOTA Coding Agents Benchmarks</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>free_text</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Short free-text field: breaking changes, important patterns, new capabilities, relevance to agentic workflows, implications for research platforms. This is where institutional knowledge accumulates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>Discovery Date</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Knowledgebase; Deprecated; SOTA Coding Agents Benchmarks</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Date this resource first entered the VT Radar.</t>
         </is>
@@ -4585,7 +4489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6161,66 +6065,168 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Maturity Level</t>
+          <t>ALAF Checklist Mapping</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Emerging</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>FFB7E1CD</t>
+          <t>Remediate Oversharing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Item (1): audit and tighten every mechanism that can grant access to the data, before the agent gets it.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Maturity Level</t>
+          <t>ALAF Checklist Mapping</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>FFFFE599</t>
+          <t>Deidentify Data</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Item (2): find and remove or hide sensitive information in the data before agents can reach it.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Maturity Level</t>
+          <t>ALAF Checklist Mapping</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Mature</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>FFA4C2F4</t>
+          <t>Agent Manifesto</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Item (3): the written rules governing agents, which they must read before tasks touching new data.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>ALAF Checklist Mapping</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Runtime PII Screening</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Item (4): a check between the agent and each new data source, with findings written where the agent cannot read them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ALAF Checklist Mapping</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Human Approval Gate</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Item (5): a named human must approve consequential actions, and the agent cannot bypass the gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ALAF Checklist Mapping</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Provenance and Reversibility</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Item (6): a record of what the agent did and who approved it, plus the ability to undo it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
           <t>Maturity Level</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>FFB7E1CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Maturity Level</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>FFFFE599</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Maturity Level</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>FFA4C2F4</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Maturity Level</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
         <is>
           <t>Deprecated</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>FFDD7E6B</t>
         </is>
@@ -6241,7 +6247,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="4"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
added ALAF-Checklist and added ALAF Checklist Mapping column to VT Radar
</commit_message>
<xml_diff>
--- a/data/VANTAGE-Technology-Radar.xlsx
+++ b/data/VANTAGE-Technology-Radar.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="19090" yWindow="-690" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Knowledgebase" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,16 +14,16 @@
     <sheet name="Standards" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,11 +32,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <color rgb="FF0563C1"/>
+      <sz val="11"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,24 +68,43 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="59">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFD9D2E9"/>
-          <bgColor rgb="FFD9D2E9"/>
+          <fgColor rgb="FFDD7E6B"/>
+          <bgColor rgb="FFDD7E6B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA4C2F4"/>
+          <bgColor rgb="FFA4C2F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFE599"/>
+          <bgColor rgb="FFFFE599"/>
         </patternFill>
       </fill>
     </dxf>
@@ -89,8 +119,88 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFA4C2F4"/>
-          <bgColor rgb="FFA4C2F4"/>
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB6D7A8"/>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAD1DC"/>
+          <bgColor rgb="FFEAD1DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCFE2F3"/>
+          <bgColor rgb="FFCFE2F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE5CD"/>
+          <bgColor rgb="FFFCE5CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD0E0E3"/>
+          <bgColor rgb="FFD0E0E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC9DAF8"/>
+          <bgColor rgb="FFC9DAF8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFE599"/>
+          <bgColor rgb="FFFFE599"/>
         </patternFill>
       </fill>
     </dxf>
@@ -105,8 +215,136 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFA4C2F4"/>
+          <bgColor rgb="FFA4C2F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9D2E9"/>
+          <bgColor rgb="FFD9D2E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDD7E6B"/>
+          <bgColor rgb="FFDD7E6B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA4C2F4"/>
+          <bgColor rgb="FFA4C2F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFE599"/>
           <bgColor rgb="FFFFE599"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB6D7A8"/>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAD1DC"/>
+          <bgColor rgb="FFEAD1DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCFE2F3"/>
+          <bgColor rgb="FFCFE2F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE5CD"/>
+          <bgColor rgb="FFFCE5CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD0E0E3"/>
+          <bgColor rgb="FFD0E0E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC9DAF8"/>
+          <bgColor rgb="FFC9DAF8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEA9999"/>
+          <bgColor rgb="FFEA9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -121,8 +359,136 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFD9EAD3"/>
-          <bgColor rgb="FFD9EAD3"/>
+          <fgColor rgb="FFFFE599"/>
+          <bgColor rgb="FFFFE599"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB4A7D6"/>
+          <bgColor rgb="FFB4A7D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA4C2F4"/>
+          <bgColor rgb="FFA4C2F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9D2E9"/>
+          <bgColor rgb="FFD9D2E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDD7E6B"/>
+          <bgColor rgb="FFDD7E6B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFA4C2F4"/>
+          <bgColor rgb="FFA4C2F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFE599"/>
+          <bgColor rgb="FFFFE599"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE06666"/>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB6D7A8"/>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEAD1DC"/>
+          <bgColor rgb="FFEAD1DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCFE2F3"/>
+          <bgColor rgb="FFCFE2F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE5CD"/>
+          <bgColor rgb="FFFCE5CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD0E0E3"/>
+          <bgColor rgb="FFD0E0E3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC9DAF8"/>
+          <bgColor rgb="FFC9DAF8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -137,64 +503,56 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFC9DAF8"/>
-          <bgColor rgb="FFC9DAF8"/>
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFD0E0E3"/>
-          <bgColor rgb="FFD0E0E3"/>
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFCE5CD"/>
-          <bgColor rgb="FFFCE5CD"/>
+          <fgColor rgb="FFFFE599"/>
+          <bgColor rgb="FFFFE599"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFCFE2F3"/>
-          <bgColor rgb="FFCFE2F3"/>
+          <fgColor rgb="FFB4A7D6"/>
+          <bgColor rgb="FFB4A7D6"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFEAD1DC"/>
-          <bgColor rgb="FFEAD1DC"/>
+          <fgColor rgb="FFA4C2F4"/>
+          <bgColor rgb="FFA4C2F4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFB6D7A8"/>
-          <bgColor rgb="FFB6D7A8"/>
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE06666"/>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDD7E6B"/>
-          <bgColor rgb="FFDD7E6B"/>
+          <fgColor rgb="FFD9D2E9"/>
+          <bgColor rgb="FFD9D2E9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -564,7 +922,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="36.5703125" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -757,12 +1115,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Data Director</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/document/d/1mu1_U1cWqn1aP3vtW83JnX5-aGhzM49K/edit</t>
+          <t>RDA Data Director Agentic AI Blueprint</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rd-alliance.org/groups/data-director-agentic-ai-blueprint/outputs/data-director-agentic-ai-tool-blueprint/</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -771,7 +1129,7 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>46168</v>
+        <v>46266</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -784,7 +1142,7 @@
         </is>
       </c>
       <c r="H3" s="3" t="n">
-        <v>46168</v>
+        <v>46266</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -1788,12 +2146,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Anthropic Safety Guidelines</t>
+          <t>Anthropic Security Safeguards</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>https://docs.anthropic.com/en/docs/safety</t>
+          <t>https://code.claude.com/docs/en/security</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1801,11 +2159,22 @@
           <t>Anthropic</t>
         </is>
       </c>
+      <c r="E19" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Paty Buendia</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
+      <c r="H19" s="3" t="n">
+        <v>46266</v>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>Documentation</t>
@@ -1823,7 +2192,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Agent Manifesto</t>
+          <t>Agent Manifesto;Zero Data Retention</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2892,70 +3261,70 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E34">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="18">
       <formula>E2&gt;=DATE(2026,5,9)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K34">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
       <formula>"Documentation"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"API Reference"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="15">
       <formula>"Specification"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
       <formula>"Whitepaper"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="13">
       <formula>"Scientific Literature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="12">
       <formula>"Governance Guidance"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="11">
       <formula>"Security Guidance &amp; Resources"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="10">
       <formula>"Reference Architecture"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"Container Registry"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
       <formula>"Enterprise Control Interface"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
       <formula>"Inference Framework"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="6">
       <formula>"Local Application Sandbox"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
       <formula>"Github Code Repository"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="4">
       <formula>"Benchmark Collection"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M34">
-    <cfRule type="expression" priority="16" dxfId="1">
+    <cfRule type="expression" priority="16" dxfId="3">
       <formula>LEN(TRIM(M2))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2:P34">
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="3">
       <formula>"Emerging"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
       <formula>"Research"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="1">
       <formula>"Mature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="15">
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="0">
       <formula>"Deprecated"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3146,7 +3515,14 @@
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n"/>
+      <c r="E2" s="3" t="n">
+        <v>46265</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Paty Buendia</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Paty Buendia</t>
@@ -3265,70 +3641,70 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E3">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="18">
       <formula>E2&gt;=DATE(2026,5,9)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L3">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
       <formula>"Documentation"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"API Reference"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="15">
       <formula>"Specification"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
       <formula>"Whitepaper"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="13">
       <formula>"Scientific Literature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="12">
       <formula>"Governance Guidance"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="11">
       <formula>"Security Guidance &amp; Resources"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="10">
       <formula>"Reference Architecture"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"Container Registry"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
       <formula>"Enterprise Control Interface"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
       <formula>"Inference Framework"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="6">
       <formula>"Local Application Sandbox"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
       <formula>"Github Code Repository"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="4">
       <formula>"Benchmark Collection"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N3">
-    <cfRule type="expression" priority="16" dxfId="1">
+    <cfRule type="expression" priority="16" dxfId="3">
       <formula>LEN(TRIM(N2))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:Q3">
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="3">
       <formula>"Emerging"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
       <formula>"Research"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="1">
       <formula>"Mature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="20" operator="equal" dxfId="15">
+    <cfRule type="cellIs" priority="20" operator="equal" dxfId="0">
       <formula>"Deprecated"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3848,65 +4224,65 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E8">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="18">
       <formula>E2&gt;=DATE(2026,5,9)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K8">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
       <formula>"Documentation"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
       <formula>"API Reference"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="15">
       <formula>"Specification"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="2">
       <formula>"Whitepaper"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="13">
       <formula>"Scientific Literature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="12">
       <formula>"Governance Guidance"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="11">
       <formula>"Security Guidance &amp; Resources"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="10">
       <formula>"Reference Architecture"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"Container Registry"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="8">
       <formula>"Enterprise Control Interface"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="7">
       <formula>"Inference Framework"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="12">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="6">
       <formula>"Local Application Sandbox"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="13">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
       <formula>"Github Code Repository"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="4">
       <formula>"Benchmark Collection"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N8">
-    <cfRule type="cellIs" priority="16" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="3">
       <formula>"Emerging"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="2">
       <formula>"Research"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="1">
       <formula>"Mature"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="15">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="0">
       <formula>"Deprecated"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3934,8 +4310,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="80" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -4489,7 +4864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6075,7 +6450,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Item (1): audit and tighten every mechanism that can grant access to the data, before the agent gets it.</t>
+          <t>Audit and tighten every mechanism that can grant access to the data, before the agent gets it.</t>
         </is>
       </c>
     </row>
@@ -6092,7 +6467,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Item (2): find and remove or hide sensitive information in the data before agents can reach it.</t>
+          <t>Find and remove or hide sensitive information in the data before agents can reach it.</t>
         </is>
       </c>
     </row>
@@ -6109,7 +6484,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Item (3): the written rules governing agents, which they must read before tasks touching new data.</t>
+          <t>The written rules governing agents, which they must read before tasks touching new data.</t>
         </is>
       </c>
     </row>
@@ -6126,7 +6501,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Item (4): a check between the agent and each new data source, with findings written where the agent cannot read them.</t>
+          <t>A check between the agent and each new data source, with findings written where the agent cannot read them.</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6518,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Item (5): a named human must approve consequential actions, and the agent cannot bypass the gate.</t>
+          <t>A named human must approve consequential actions, and the agent cannot bypass the gate.</t>
         </is>
       </c>
     </row>
@@ -6160,24 +6535,24 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Item (6): a record of what the agent did and who approved it, plus the ability to undo it.</t>
+          <t>A record of what the agent did and who approved it, plus the ability to undo it.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Maturity Level</t>
+          <t>ALAF Checklist Mapping</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Emerging</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>FFB7E1CD</t>
+          <t>Zero Data Retention</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Third-party AI APIs configured for zero data retention, with the prompt caching TTL checked separately.</t>
         </is>
       </c>
     </row>
@@ -6189,12 +6564,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Emerging</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>FFFFE599</t>
+          <t>FFB7E1CD</t>
         </is>
       </c>
     </row>
@@ -6206,12 +6581,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Mature</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>FFA4C2F4</t>
+          <t>FFFFE599</t>
         </is>
       </c>
     </row>
@@ -6223,10 +6598,27 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>Mature</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>FFA4C2F4</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Maturity Level</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>Deprecated</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>FFDD7E6B</t>
         </is>
@@ -6247,9 +6639,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="2" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>

</xml_diff>